<commit_message>
final før første innlevering
</commit_message>
<xml_diff>
--- a/MPLS_YAY/demo.xlsx
+++ b/MPLS_YAY/demo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yonat\Videos\INI\MPLS_YAY\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64622152-FFE2-4129-9904-1FE4B15E5C5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C97A853-CC1E-42CA-8A95-12320B5D3AAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Site 1 (HUB)" sheetId="1" r:id="rId1"/>
@@ -35,8 +35,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="97">
   <si>
     <t>site</t>
   </si>
@@ -129,9 +151,6 @@
   </si>
   <si>
     <t>MGMT</t>
-  </si>
-  <si>
-    <t>255.255.0.0</t>
   </si>
   <si>
     <t>INET</t>
@@ -491,7 +510,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -509,7 +528,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -573,11 +591,43 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="149">
+  <dxfs count="131">
+    <dxf>
+      <font>
+        <u val="none"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <u val="none"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <font>
         <color theme="1"/>
@@ -643,126 +693,6 @@
     <dxf>
       <font>
         <sz val="11"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
       </font>
     </dxf>
     <dxf>
@@ -1399,126 +1329,6 @@
     <dxf>
       <font>
         <sz val="11"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
       </font>
     </dxf>
     <dxf>
@@ -1915,213 +1725,243 @@
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="brukernavn"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="passord"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="vty_lines"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="secret" dataDxfId="88"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="tacacs_key" dataDxfId="87"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="DHCP" dataDxfId="86"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="dns_servers" dataDxfId="85"/>
-    <tableColumn id="11" xr3:uid="{A73DBE03-6D2F-4B6E-9364-0ACF9BE031A7}" name="tacacs_server_ip" dataDxfId="84"/>
-    <tableColumn id="12" xr3:uid="{610238BB-82C8-435E-9688-053D824B1B9E}" name="syslog_server_ip" dataDxfId="83"/>
-    <tableColumn id="13" xr3:uid="{E7D67AED-C401-4BA3-8148-89AED6E825C5}" name="urpf_mode" dataDxfId="82"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="secret" dataDxfId="82"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="tacacs_key" dataDxfId="81"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="DHCP" dataDxfId="80"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="dns_servers" dataDxfId="79"/>
+    <tableColumn id="11" xr3:uid="{A73DBE03-6D2F-4B6E-9364-0ACF9BE031A7}" name="tacacs_server_ip" dataDxfId="78"/>
+    <tableColumn id="12" xr3:uid="{610238BB-82C8-435E-9688-053D824B1B9E}" name="syslog_server_ip" dataDxfId="77"/>
+    <tableColumn id="13" xr3:uid="{E7D67AED-C401-4BA3-8148-89AED6E825C5}" name="urpf_mode" dataDxfId="76"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="29" xr:uid="{00000000-000C-0000-FFFF-FFFF09000000}" name="Tabell13192530" displayName="Tabell13192530" ref="A21:G22" dataDxfId="30">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="29" xr:uid="{00000000-000C-0000-FFFF-FFFF09000000}" name="Tabell13192530" displayName="Tabell13192530" ref="A21:G22" dataDxfId="24">
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0900-000001000000}" name="site" dataDxfId="29">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0900-000001000000}" name="site" dataDxfId="23">
       <calculatedColumnFormula>A2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0900-000004000000}" name="brukernavn" dataDxfId="28"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0900-000005000000}" name="passord" dataDxfId="27"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0900-000003000000}" name="vty_lines" dataDxfId="26"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0900-000002000000}" name="secret" dataDxfId="25"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0900-000006000000}" name="etherchan_num" dataDxfId="24"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0900-000007000000}" name="span_mode" dataDxfId="23"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0900-000004000000}" name="brukernavn" dataDxfId="22"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0900-000005000000}" name="passord" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0900-000003000000}" name="vty_lines" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0900-000002000000}" name="secret" dataDxfId="19"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0900-000006000000}" name="etherchan_num" dataDxfId="18"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0900-000007000000}" name="span_mode" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF0A000000}" name="Tabell2" displayName="Tabell2" ref="A4:K8" dataDxfId="22">
-  <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0A00-000001000000}" name="vrf" dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0A00-000002000000}" name="vlan" dataDxfId="20"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0A00-000003000000}" name="interface" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0A00-000004000000}" name="nett id" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0A00-000005000000}" name="gateway" dataDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0A00-000006000000}" name="mask" dataDxfId="16"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0A00-000007000000}" name="address min" dataDxfId="15"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0A00-000008000000}" name="address max" dataDxfId="14"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0A00-000009000000}" name="antall-res" dataDxfId="13"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0A00-00000A000000}" name="pri-afxx" dataDxfId="12"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0A00-00000B000000}" name="pri-1-10" dataDxfId="11"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="31" xr:uid="{00000000-000C-0000-FFFF-FFFF0B000000}" name="Tabell161824282532" displayName="Tabell161824282532" ref="A24:L25" totalsRowShown="0">
+  <tableColumns count="12">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0B00-000001000000}" name="SW" dataDxfId="16">
+      <calculatedColumnFormula>(ROW())-(ROW()-1)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0B00-000002000000}" name="MGMT Vlan" dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0B00-000003000000}" name="MGMT ip" dataDxfId="14">
+      <calculatedColumnFormula>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A25)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0B00-000004000000}" name="gateway" dataDxfId="13">
+      <calculatedColumnFormula>$E$5</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0B00-000005000000}" name="mask" dataDxfId="12">
+      <calculatedColumnFormula>$F$5</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0B00-00000A000000}" name="num_ports_tot" dataDxfId="11"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0B00-00000B000000}" name="skiped_ports" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0B00-000006000000}" name="num_downlink" dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0B00-000007000000}" name="vlan-antall" dataDxfId="8"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0B00-000008000000}" name="intf_prefix" dataDxfId="7"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0B00-000009000000}" name="num_port_ledig" dataDxfId="6">
+      <calculatedColumnFormula>IF($A25=1,F25-G25-H25*$F$22-2-IF(OR(UPPER($G$22)="SPAN",UPPER($G$22)="RSPAN"),1,0),F25-G25-(1+H25)*$F$22-1)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0B00-00000C000000}" name="MONITORING ip">
+      <calculatedColumnFormula>10&amp;"."&amp;(50+$A$2)&amp;"."&amp;0&amp;"."&amp;(A25+1)</calculatedColumnFormula>
+    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="31" xr:uid="{00000000-000C-0000-FFFF-FFFF0B000000}" name="Tabell161824282532" displayName="Tabell161824282532" ref="A24:L25" totalsRowShown="0">
-  <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0B00-000001000000}" name="SW" dataDxfId="10">
-      <calculatedColumnFormula>(ROW())-(ROW()-1)</calculatedColumnFormula>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6D5A02AD-2CA6-4912-AA9B-3C6CC47A8FA5}" name="Tabell62" displayName="Tabell62" ref="A4:K8">
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{47B3C139-1692-4650-99C8-309AED464DC1}" name="vrf"/>
+    <tableColumn id="2" xr3:uid="{D62DD834-E0BB-4909-89A0-12F620F06BC8}" name="vlan"/>
+    <tableColumn id="3" xr3:uid="{345E6AA5-B02C-4C04-BAC7-4DC8E61BBD06}" name="interface"/>
+    <tableColumn id="4" xr3:uid="{24F3CFC8-48FF-467B-A0AD-4AA8452B8BE1}" name="nett id" dataDxfId="3">
+      <calculatedColumnFormula>10&amp;"."&amp;($A$2)&amp;"."&amp;$B5&amp;"."&amp;0</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0B00-000002000000}" name="MGMT Vlan" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0B00-000003000000}" name="MGMT ip" dataDxfId="8">
-      <calculatedColumnFormula>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A25)</calculatedColumnFormula>
+    <tableColumn id="5" xr3:uid="{7491CD15-10DB-4123-92F7-6CEB0CF5B9A8}" name="gateway">
+      <calculatedColumnFormula>LEFT(D5,LEN(D5)-1)&amp;"1"</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0B00-000004000000}" name="gateway" dataDxfId="7">
-      <calculatedColumnFormula>$E$5</calculatedColumnFormula>
+    <tableColumn id="6" xr3:uid="{22BAF84C-332E-43D7-ABD2-6170B30E36FA}" name="mask"/>
+    <tableColumn id="7" xr3:uid="{0F964A11-FF57-46EC-961F-CDB26E5E1483}" name="address min">
+      <calculatedColumnFormula array="1">_xlfn.LET(
+_xlpm.net,SUM(--_xlfn.TEXTSPLIT(Tabell62[[#This Row],[nett id]],".")*{16777216,65536,256,1}),
+_xlpm.addr,_xlpm.net+1,
+_xlfn.TEXTJOIN(".",TRUE,MOD(QUOTIENT(_xlpm.addr,{16777216,65536,256,1}),256))
+)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0B00-000005000000}" name="mask" dataDxfId="6">
-      <calculatedColumnFormula>$F$5</calculatedColumnFormula>
+    <tableColumn id="8" xr3:uid="{391A005D-CAFC-426C-A5F3-725914B53829}" name="address max">
+      <calculatedColumnFormula array="1">_xlfn.LET(
+_xlpm.net,SUM(--_xlfn.TEXTSPLIT(Tabell62[[#This Row],[nett id]],".")*{16777216,65536,256,1}),
+_xlpm.mask,SUM(--_xlfn.TEXTSPLIT(Tabell62[[#This Row],[mask]],".")*{16777216,65536,256,1}),
+_xlpm.addr,_xlpm.net+(4294967295-_xlpm.mask)-1,
+_xlfn.TEXTJOIN(".",TRUE,MOD(QUOTIENT(_xlpm.addr,{16777216,65536,256,1}),256))
+)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0B00-00000A000000}" name="num_ports_tot" dataDxfId="5"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0B00-00000B000000}" name="skiped_ports" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0B00-000006000000}" name="num_downlink" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0B00-000007000000}" name="vlan-antall" dataDxfId="2"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0B00-000008000000}" name="intf_prefix" dataDxfId="1"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0B00-000009000000}" name="num_port_ledig" dataDxfId="0">
-      <calculatedColumnFormula>IF($A25=1,F25-G25-H25*$F$22-2-IF(OR(UPPER($G$22)="SPAN",UPPER($G$22)="RSPAN"),1,0),F25-G25-(1+H25)*$F$22-1)</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0B00-00000C000000}" name="MONITORING ip"/>
+    <tableColumn id="9" xr3:uid="{9EC1882B-AF0A-44F1-BD9A-8A894B349CA3}" name="antall-res" dataDxfId="2"/>
+    <tableColumn id="10" xr3:uid="{61EDD6C0-0C78-4240-AF0C-CB240D30092C}" name="pri-afxx"/>
+    <tableColumn id="11" xr3:uid="{B63F8595-9D02-4C92-9525-FDF21F956CD6}" name="pri-1-10"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="24" xr:uid="{00000000-000C-0000-FFFF-FFFF0C000000}" name="Tabell125" displayName="Tabell125" ref="A1:L2" dataDxfId="148">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="24" xr:uid="{00000000-000C-0000-FFFF-FFFF0C000000}" name="Tabell125" displayName="Tabell125" ref="A1:L2" dataDxfId="130">
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0C00-000001000000}" name="site" dataDxfId="147"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0C00-000002000000}" name="intf_prefix" dataDxfId="146"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0C00-000003000000}" name="router-id" dataDxfId="145">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0C00-000001000000}" name="site" dataDxfId="129"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0C00-000002000000}" name="intf_prefix" dataDxfId="128"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0C00-000003000000}" name="router-id" dataDxfId="127">
       <calculatedColumnFormula>A2&amp;"."&amp;A2&amp;"."&amp;A2&amp;".0"</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0C00-000004000000}" name="brukernavn" dataDxfId="144"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0C00-000005000000}" name="passord" dataDxfId="143"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0C00-000006000000}" name="vty_lines" dataDxfId="142"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0C00-000007000000}" name="secret" dataDxfId="141"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0C00-000008000000}" name="tacacs_key" dataDxfId="140">
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0C00-000004000000}" name="brukernavn" dataDxfId="126"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0C00-000005000000}" name="passord" dataDxfId="125"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0C00-000006000000}" name="vty_lines" dataDxfId="124"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0C00-000007000000}" name="secret" dataDxfId="123"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0C00-000008000000}" name="tacacs_key" dataDxfId="122">
       <calculatedColumnFormula>'Site 1 (HUB)'!H2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0C00-000009000000}" name="dns_servers" dataDxfId="139"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0C00-00000A000000}" name="tacacs_server_ip" dataDxfId="138">
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0C00-000009000000}" name="dns_servers" dataDxfId="121"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0C00-00000A000000}" name="tacacs_server_ip" dataDxfId="120">
       <calculatedColumnFormula>'Site 1 (HUB)'!K2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0C00-00000B000000}" name="syslog_server_ip" dataDxfId="137">
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0C00-00000B000000}" name="syslog_server_ip" dataDxfId="119">
       <calculatedColumnFormula>'Site 1 (HUB)'!L2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{8F454925-3BC4-4EBB-8D3D-A7176AFC9BBB}" name="urpf_mode" dataDxfId="136"/>
+    <tableColumn id="12" xr3:uid="{8F454925-3BC4-4EBB-8D3D-A7176AFC9BBB}" name="urpf_mode" dataDxfId="118"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="25" xr:uid="{00000000-000C-0000-FFFF-FFFF0D000000}" name="Tabell326" displayName="Tabell326" ref="A10:D14" dataDxfId="135">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="25" xr:uid="{00000000-000C-0000-FFFF-FFFF0D000000}" name="Tabell326" displayName="Tabell326" ref="A10:D14" dataDxfId="117">
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0D00-000001000000}" name="vrf" dataDxfId="134"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0D00-000002000000}" name="rt" dataDxfId="133"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0D00-000003000000}" name="loopback" dataDxfId="132"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0D00-000004000000}" name="laddr" dataDxfId="131"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0D00-000001000000}" name="vrf" dataDxfId="116"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0D00-000002000000}" name="rt" dataDxfId="115"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0D00-000003000000}" name="loopback" dataDxfId="114"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0D00-000004000000}" name="laddr" dataDxfId="113"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="26" xr:uid="{00000000-000C-0000-FFFF-FFFF0E000000}" name="Tabell427" displayName="Tabell427" ref="A16:J19" dataDxfId="130">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="26" xr:uid="{00000000-000C-0000-FFFF-FFFF0E000000}" name="Tabell427" displayName="Tabell427" ref="A16:J19" dataDxfId="112">
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0E00-000001000000}" name="tunnel id" dataDxfId="129"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0E00-000002000000}" name="vrf" dataDxfId="128"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0E00-000003000000}" name="ip address" dataDxfId="127">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0E00-000001000000}" name="tunnel id" dataDxfId="111"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0E00-000002000000}" name="vrf" dataDxfId="110"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0E00-000003000000}" name="ip address" dataDxfId="109">
       <calculatedColumnFormula>172&amp;"."&amp;16&amp;"."&amp;0&amp;"."&amp;(H17+$A$2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0E00-000004000000}" name="mask" dataDxfId="126"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0E00-000005000000}" name="source" dataDxfId="125">
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0E00-000004000000}" name="mask" dataDxfId="108"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0E00-000005000000}" name="source" dataDxfId="107">
       <calculatedColumnFormula>LEFT($C$2,LEN($C$2)-1)&amp;Tabell427[[#This Row],[network-id]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0E00-000006000000}" name="destination" dataDxfId="124"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0E00-000007000000}" name="gre mode" dataDxfId="123"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0E00-000008000000}" name="network-id" dataDxfId="122"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0E00-000009000000}" name="ipsec" dataDxfId="121"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0E00-00000A000000}" name="ipsec key" dataDxfId="120"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0E00-000006000000}" name="destination" dataDxfId="106"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0E00-000007000000}" name="gre mode" dataDxfId="105"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0E00-000008000000}" name="network-id" dataDxfId="104"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0E00-000009000000}" name="ipsec" dataDxfId="103"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0E00-00000A000000}" name="ipsec key" dataDxfId="102"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="27" xr:uid="{00000000-000C-0000-FFFF-FFFF0F000000}" name="Tabell1319253028" displayName="Tabell1319253028" ref="A21:G22" dataDxfId="119">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="27" xr:uid="{00000000-000C-0000-FFFF-FFFF0F000000}" name="Tabell1319253028" displayName="Tabell1319253028" ref="A21:G22" dataDxfId="101">
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0F00-000001000000}" name="site" dataDxfId="118">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0F00-000001000000}" name="site" dataDxfId="100">
       <calculatedColumnFormula>A2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0F00-000004000000}" name="brukernavn" dataDxfId="117"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0F00-000005000000}" name="passord" dataDxfId="116"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0F00-000003000000}" name="vty_lines" dataDxfId="115"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0F00-000002000000}" name="secret" dataDxfId="114"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0F00-000006000000}" name="etherchan_num" dataDxfId="113"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0F00-000007000000}" name="span_mode" dataDxfId="112"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0F00-000004000000}" name="brukernavn" dataDxfId="99"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0F00-000005000000}" name="passord" dataDxfId="98"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0F00-000003000000}" name="vty_lines" dataDxfId="97"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0F00-000002000000}" name="secret" dataDxfId="96"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0F00-000006000000}" name="etherchan_num" dataDxfId="95"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0F00-000007000000}" name="span_mode" dataDxfId="94"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="30" xr:uid="{00000000-000C-0000-FFFF-FFFF10000000}" name="Tabell231" displayName="Tabell231" ref="A4:K8" dataDxfId="111">
-  <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-1000-000001000000}" name="vrf" dataDxfId="110"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-1000-000002000000}" name="vlan" dataDxfId="109"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-1000-000003000000}" name="interface" dataDxfId="108"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-1000-000004000000}" name="nett id" dataDxfId="107"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-1000-000005000000}" name="gateway" dataDxfId="106">
-      <calculatedColumnFormula>LEFT(D5,LEN(D5)-1)&amp;"1"</calculatedColumnFormula>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="32" xr:uid="{00000000-000C-0000-FFFF-FFFF11000000}" name="Tabell16182428253233" displayName="Tabell16182428253233" ref="A24:L25" totalsRowShown="0">
+  <tableColumns count="12">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-1100-000001000000}" name="SW" dataDxfId="93">
+      <calculatedColumnFormula>(ROW())-(ROW()-1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-1000-000006000000}" name="mask" dataDxfId="105"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-1000-000007000000}" name="address min" dataDxfId="104">
-      <calculatedColumnFormula>LEFT(D5,LEN(D5)-1)&amp;"1"</calculatedColumnFormula>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-1100-000002000000}" name="MGMT Vlan" dataDxfId="92"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-1100-000003000000}" name="MGMT ip" dataDxfId="91">
+      <calculatedColumnFormula>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A25)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-1000-000008000000}" name="address max" dataDxfId="103">
-      <calculatedColumnFormula>LEFT(D5,FIND(".",D5,FIND(".",D5)+1)-1)&amp;".255.254"</calculatedColumnFormula>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-1100-000004000000}" name="gateway" dataDxfId="90">
+      <calculatedColumnFormula>$E$5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-1000-000009000000}" name="antall-res" dataDxfId="102"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-1000-00000A000000}" name="pri-afxx" dataDxfId="101"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-1000-00000B000000}" name="pri-1-10" dataDxfId="100"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-1100-000005000000}" name="mask" dataDxfId="89">
+      <calculatedColumnFormula>$F$5</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-1100-00000A000000}" name="num_ports_tot" dataDxfId="88"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-1100-00000B000000}" name="skiped_ports" dataDxfId="87"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-1100-000006000000}" name="num_downlink" dataDxfId="86"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-1100-000007000000}" name="vlan-antall" dataDxfId="85"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-1100-000008000000}" name="intf_prefix" dataDxfId="84"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-1100-000009000000}" name="num_port_ledig" dataDxfId="83">
+      <calculatedColumnFormula>IF($A25=1,F25-G25-H25*$F$22-2-IF(OR($G$22="ERSPAN",$G$22="SPAN",$G$22="RSPAN"),1,0),F25-G25-(1+H25)*$F$22-1)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-1100-00000C000000}" name="MONITORING ip"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="32" xr:uid="{00000000-000C-0000-FFFF-FFFF11000000}" name="Tabell16182428253233" displayName="Tabell16182428253233" ref="A24:L25" totalsRowShown="0">
-  <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-1100-000001000000}" name="SW" dataDxfId="99">
-      <calculatedColumnFormula>(ROW())-(ROW()-1)</calculatedColumnFormula>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{46FFD175-B94A-4F33-8F16-6557AA1812D1}" name="Tabell628" displayName="Tabell628" ref="A4:K8">
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{56D4B413-3CC2-4741-8FB2-EB562529AEFD}" name="vrf"/>
+    <tableColumn id="2" xr3:uid="{2563D53E-B705-4025-8974-EB012818C3A1}" name="vlan"/>
+    <tableColumn id="3" xr3:uid="{DDFF1A20-AA13-40E0-81C7-C23FF1C01637}" name="interface"/>
+    <tableColumn id="4" xr3:uid="{0FD0195F-E29B-4997-B5EF-665D39C2D2F7}" name="nett id" dataDxfId="1">
+      <calculatedColumnFormula>10&amp;"."&amp;($A$2)&amp;"."&amp;$B5&amp;"."&amp;0</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-1100-000002000000}" name="MGMT Vlan" dataDxfId="98"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-1100-000003000000}" name="MGMT ip" dataDxfId="97">
-      <calculatedColumnFormula>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A25)</calculatedColumnFormula>
+    <tableColumn id="5" xr3:uid="{10FC9A73-5C94-4AE7-8C2C-D8539C3A5C31}" name="gateway">
+      <calculatedColumnFormula>LEFT(D5,LEN(D5)-1)&amp;"1"</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-1100-000004000000}" name="gateway" dataDxfId="96">
-      <calculatedColumnFormula>$E$5</calculatedColumnFormula>
+    <tableColumn id="6" xr3:uid="{D21B1B63-EA2B-4FF7-A5B7-8EA2875C5141}" name="mask"/>
+    <tableColumn id="7" xr3:uid="{8C3295FB-EB91-4A27-9F82-8A84EFFD5BF3}" name="address min">
+      <calculatedColumnFormula array="1">_xlfn.LET(
+_xlpm.net,SUM(--_xlfn.TEXTSPLIT(Tabell628[[#This Row],[nett id]],".")*{16777216,65536,256,1}),
+_xlpm.addr,_xlpm.net+1,
+_xlfn.TEXTJOIN(".",TRUE,MOD(QUOTIENT(_xlpm.addr,{16777216,65536,256,1}),256))
+)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-1100-000005000000}" name="mask" dataDxfId="95">
-      <calculatedColumnFormula>$F$5</calculatedColumnFormula>
+    <tableColumn id="8" xr3:uid="{2F92A364-3126-4657-9B3E-F6399F54C980}" name="address max">
+      <calculatedColumnFormula array="1">_xlfn.LET(
+_xlpm.net,SUM(--_xlfn.TEXTSPLIT(Tabell628[[#This Row],[nett id]],".")*{16777216,65536,256,1}),
+_xlpm.mask,SUM(--_xlfn.TEXTSPLIT(Tabell628[[#This Row],[mask]],".")*{16777216,65536,256,1}),
+_xlpm.addr,_xlpm.net+(4294967295-_xlpm.mask)-1,
+_xlfn.TEXTJOIN(".",TRUE,MOD(QUOTIENT(_xlpm.addr,{16777216,65536,256,1}),256))
+)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-1100-00000A000000}" name="num_ports_tot" dataDxfId="94"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-1100-00000B000000}" name="skiped_ports" dataDxfId="93"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-1100-000006000000}" name="num_downlink" dataDxfId="92"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-1100-000007000000}" name="vlan-antall" dataDxfId="91"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-1100-000008000000}" name="intf_prefix" dataDxfId="90"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-1100-000009000000}" name="num_port_ledig" dataDxfId="89">
-      <calculatedColumnFormula>IF($A25=1,F25-G25-H25*$F$22-2-IF(OR($G$22="ERSPAN",$G$22="SPAN",$G$22="RSPAN"),1,0),F25-G25-(1+H25)*$F$22-1)</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-1100-00000C000000}" name="MONITORING ip"/>
+    <tableColumn id="9" xr3:uid="{F1862C6A-FC54-4E31-BF6B-5DAFB122444E}" name="antall-res" dataDxfId="0"/>
+    <tableColumn id="10" xr3:uid="{90961B88-7A7F-4994-8927-A856A56857A2}" name="pri-afxx"/>
+    <tableColumn id="11" xr3:uid="{7178CB93-6875-42D2-A7A7-EBE1AB7EEDAB}" name="pri-1-10"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2146,12 +1986,27 @@
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="vrf"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="vlan"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="interface"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="nett id"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="nett id" dataDxfId="4">
+      <calculatedColumnFormula>10&amp;"."&amp;($A$2)&amp;"."&amp;$B5&amp;"."&amp;0</calculatedColumnFormula>
+    </tableColumn>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="gateway"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="mask"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="address min"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="address max"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="antall-res" dataDxfId="81"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="address min">
+      <calculatedColumnFormula array="1">_xlfn.LET(
+_xlpm.net,SUM(--_xlfn.TEXTSPLIT(Tabell6[[#This Row],[nett id]],".")*{16777216,65536,256,1}),
+_xlpm.addr,_xlpm.net+1,
+_xlfn.TEXTJOIN(".",TRUE,MOD(QUOTIENT(_xlpm.addr,{16777216,65536,256,1}),256))
+)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="address max">
+      <calculatedColumnFormula array="1">_xlfn.LET(
+_xlpm.net,SUM(--_xlfn.TEXTSPLIT(Tabell6[[#This Row],[nett id]],".")*{16777216,65536,256,1}),
+_xlpm.mask,SUM(--_xlfn.TEXTSPLIT(Tabell6[[#This Row],[mask]],".")*{16777216,65536,256,1}),
+_xlpm.addr,_xlpm.net+(4294967295-_xlpm.mask)-1,
+_xlfn.TEXTJOIN(".",TRUE,MOD(QUOTIENT(_xlpm.addr,{16777216,65536,256,1}),256))
+)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="antall-res" dataDxfId="75"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="pri-afxx"/>
     <tableColumn id="11" xr3:uid="{00000000-0010-0000-0100-00000B000000}" name="pri-1-10"/>
   </tableColumns>
@@ -2163,7 +2018,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Tabell7" displayName="Tabell7" ref="A10:D14">
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="vrf"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="rt" dataDxfId="80"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="rt" dataDxfId="74"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="loopback"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="laddr">
       <calculatedColumnFormula>$A$2&amp;"."&amp;$A$2&amp;"."&amp;$A$2&amp;"."&amp;(C11)</calculatedColumnFormula>
@@ -2178,11 +2033,11 @@
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="tunnel id"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="vrf"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="ip address">
-      <calculatedColumnFormula>172&amp;"."&amp;16&amp;"."&amp;0&amp;"."&amp;(H17+$A$2)</calculatedColumnFormula>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="ip address" dataDxfId="5">
+      <calculatedColumnFormula>172&amp;"."&amp;16&amp;"."&amp;$H17&amp;"."&amp;($A$2)</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0300-000004000000}" name="mask"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="source" dataDxfId="79">
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="source" dataDxfId="73">
       <calculatedColumnFormula>LEFT($C$2,LEN($C$2)-1)&amp;Tabell427[[#This Row],[network-id]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0300-000006000000}" name="destination"/>
@@ -2196,17 +2051,17 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Tabell131921" displayName="Tabell131921" ref="A21:G22" dataDxfId="78">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Tabell131921" displayName="Tabell131921" ref="A21:G22" dataDxfId="72">
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="site" dataDxfId="77">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="site" dataDxfId="71">
       <calculatedColumnFormula>A2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="brukernavn" dataDxfId="76"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" name="passord" dataDxfId="75"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0400-000005000000}" name="vty_lines" dataDxfId="74"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="secret" dataDxfId="73"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0400-000006000000}" name="etherchan_num" dataDxfId="72"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0400-000007000000}" name="span_mode" dataDxfId="71"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="brukernavn" dataDxfId="70"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" name="passord" dataDxfId="69"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0400-000005000000}" name="vty_lines" dataDxfId="68"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="secret" dataDxfId="67"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0400-000006000000}" name="etherchan_num" dataDxfId="66"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0400-000007000000}" name="span_mode" dataDxfId="65"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2215,25 +2070,25 @@
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="Tabell1618242825" displayName="Tabell1618242825" ref="A24:L26" totalsRowShown="0">
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="SW" dataDxfId="70">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="SW" dataDxfId="64">
       <calculatedColumnFormula>(ROW())-(ROW()-1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="MGMT Vlan" dataDxfId="69"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0500-000003000000}" name="MGMT ip" dataDxfId="68">
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="MGMT Vlan" dataDxfId="63"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0500-000003000000}" name="MGMT ip" dataDxfId="62">
       <calculatedColumnFormula>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A25)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" name="gateway" dataDxfId="67">
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" name="gateway" dataDxfId="61">
       <calculatedColumnFormula>$E$5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0500-000005000000}" name="mask" dataDxfId="66">
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0500-000005000000}" name="mask" dataDxfId="60">
       <calculatedColumnFormula>$F$5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0500-00000A000000}" name="num_ports_tot" dataDxfId="65"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0500-00000B000000}" name="skiped_ports" dataDxfId="64"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0500-000006000000}" name="num_downlink" dataDxfId="63"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0500-000007000000}" name="vlan-antall" dataDxfId="62"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0500-000008000000}" name="intf_prefix" dataDxfId="61"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0500-000009000000}" name="num_port_ledig" dataDxfId="60">
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0500-00000A000000}" name="num_ports_tot" dataDxfId="59"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0500-00000B000000}" name="skiped_ports" dataDxfId="58"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0500-000006000000}" name="num_downlink" dataDxfId="57"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0500-000007000000}" name="vlan-antall" dataDxfId="56"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0500-000008000000}" name="intf_prefix" dataDxfId="55"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0500-000009000000}" name="num_port_ledig" dataDxfId="54">
       <calculatedColumnFormula>IF($A25=1,F25-G25-H25*$F$22-2-IF(OR(UPPER($G$22)="SPAN", UPPER($G$22)="ERSPAN",UPPER($G$22)="RSPAN"),1,0),F25-G25-(1+H25)*$F$22-1)</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="12" xr3:uid="{00000000-0010-0000-0500-00000C000000}" name="MONITORING ip"/>
@@ -2243,26 +2098,26 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="Tabell1" displayName="Tabell1" ref="A1:L2" dataDxfId="59">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="Tabell1" displayName="Tabell1" ref="A1:L2" dataDxfId="53">
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" name="site" dataDxfId="58"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" name="intf_prefix" dataDxfId="57"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0600-000003000000}" name="router-id" dataDxfId="56"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0600-000004000000}" name="brukernavn" dataDxfId="55"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0600-000005000000}" name="passord" dataDxfId="54"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0600-000006000000}" name="vty_lines" dataDxfId="53"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0600-000007000000}" name="secret" dataDxfId="52"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0600-000008000000}" name="tacacs_key" dataDxfId="51">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" name="site" dataDxfId="52"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" name="intf_prefix" dataDxfId="51"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0600-000003000000}" name="router-id" dataDxfId="50"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0600-000004000000}" name="brukernavn" dataDxfId="49"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0600-000005000000}" name="passord" dataDxfId="48"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0600-000006000000}" name="vty_lines" dataDxfId="47"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0600-000007000000}" name="secret" dataDxfId="46"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0600-000008000000}" name="tacacs_key" dataDxfId="45">
       <calculatedColumnFormula>'Site 1 (HUB)'!H2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0600-000009000000}" name="dns_servers" dataDxfId="50"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0600-00000A000000}" name="tacacs_server_ip" dataDxfId="49">
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0600-000009000000}" name="dns_servers" dataDxfId="44"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0600-00000A000000}" name="tacacs_server_ip" dataDxfId="43">
       <calculatedColumnFormula>'Site 1 (HUB)'!K2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0600-00000B000000}" name="syslog_server_ip" dataDxfId="48">
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0600-00000B000000}" name="syslog_server_ip" dataDxfId="42">
       <calculatedColumnFormula>'Site 1 (HUB)'!L2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{C0C3F1E4-EA14-4BE7-8B57-054084352EF9}" name="urpf_mode" dataDxfId="47">
+    <tableColumn id="12" xr3:uid="{C0C3F1E4-EA14-4BE7-8B57-054084352EF9}" name="urpf_mode" dataDxfId="41">
       <calculatedColumnFormula>'Site 1 (HUB)'!M2</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2271,34 +2126,34 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="Tabell3" displayName="Tabell3" ref="A10:D14" dataDxfId="46">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="Tabell3" displayName="Tabell3" ref="A10:D14" dataDxfId="40">
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0700-000001000000}" name="vrf" dataDxfId="45"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="rt" dataDxfId="44"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0700-000003000000}" name="loopback" dataDxfId="43"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0700-000004000000}" name="laddr" dataDxfId="42"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0700-000001000000}" name="vrf" dataDxfId="39"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="rt" dataDxfId="38"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0700-000003000000}" name="loopback" dataDxfId="37"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0700-000004000000}" name="laddr" dataDxfId="36"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{00000000-000C-0000-FFFF-FFFF08000000}" name="Tabell4" displayName="Tabell4" ref="A16:J19" dataDxfId="41">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{00000000-000C-0000-FFFF-FFFF08000000}" name="Tabell4" displayName="Tabell4" ref="A16:J19" dataDxfId="35">
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0800-000001000000}" name="tunnel id" dataDxfId="40"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0800-000002000000}" name="vrf" dataDxfId="39"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0800-000003000000}" name="ip address" dataDxfId="38">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0800-000001000000}" name="tunnel id" dataDxfId="34"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0800-000002000000}" name="vrf" dataDxfId="33"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0800-000003000000}" name="ip address" dataDxfId="32">
       <calculatedColumnFormula>172&amp;"."&amp;16&amp;"."&amp;0&amp;"."&amp;(H17+$A$2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0800-000004000000}" name="mask" dataDxfId="37"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0800-000005000000}" name="source" dataDxfId="36">
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0800-000004000000}" name="mask" dataDxfId="31"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0800-000005000000}" name="source" dataDxfId="30">
       <calculatedColumnFormula>LEFT($C$2,LEN($C$2)-1)&amp;Tabell427[[#This Row],[network-id]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0800-000006000000}" name="destination" dataDxfId="35"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0800-000007000000}" name="gre mode" dataDxfId="34"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0800-000008000000}" name="network-id" dataDxfId="33"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0800-000009000000}" name="ipsec" dataDxfId="32"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0800-00000A000000}" name="ipsec key" dataDxfId="31"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0800-000006000000}" name="destination" dataDxfId="29"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0800-000007000000}" name="gre mode" dataDxfId="28"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0800-000008000000}" name="network-id" dataDxfId="27"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0800-000009000000}" name="ipsec" dataDxfId="26"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0800-00000A000000}" name="ipsec key" dataDxfId="25"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2505,7 +2360,7 @@
     <col min="1" max="1" width="10.7109375" customWidth="1"/>
     <col min="2" max="2" width="13" customWidth="1"/>
     <col min="3" max="3" width="66" customWidth="1"/>
-    <col min="4" max="4" width="12.28515625" customWidth="1"/>
+    <col min="4" max="4" width="14.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="66" customWidth="1"/>
     <col min="6" max="6" width="15.85546875" customWidth="1"/>
     <col min="7" max="7" width="66" customWidth="1"/>
@@ -2544,17 +2399,17 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="30" t="s">
+      <c r="J1" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="31" t="s">
+      <c r="K1" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="31" t="s">
+      <c r="L1" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="32" t="s">
-        <v>68</v>
+      <c r="M1" s="31" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -2586,17 +2441,17 @@
       <c r="I2" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="J2" s="13" t="s">
+      <c r="J2" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="K2" s="19" t="s">
+      <c r="K2" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="L2" s="19" t="s">
+      <c r="L2" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="M2" s="19" t="s">
-        <v>69</v>
+      <c r="M2" s="18" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2637,121 +2492,148 @@
       <c r="I4" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="J4" s="7" t="s">
+      <c r="J4" s="32" t="s">
         <v>28</v>
       </c>
-      <c r="K4" s="7" t="s">
+      <c r="K4" s="32" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B5" s="9">
+      <c r="B5" s="8">
         <v>10</v>
       </c>
-      <c r="C5" s="8">
+      <c r="C5" s="7">
         <v>0</v>
       </c>
-      <c r="D5" s="8" t="str">
-        <f>10&amp;"."&amp;(B5+A2)&amp;"."&amp;0&amp;"."&amp;0</f>
-        <v>10.11.0.0</v>
-      </c>
-      <c r="E5" s="8" t="str">
-        <f t="shared" ref="E5:E7" si="0">LEFT(D5,LEN(D5)-1)&amp;"1"</f>
-        <v>10.11.0.1</v>
-      </c>
-      <c r="F5" s="8" t="s">
+      <c r="D5" s="7" t="str">
+        <f t="shared" ref="D5:D8" si="0">10&amp;"."&amp;($A$2)&amp;"."&amp;$B5&amp;"."&amp;0</f>
+        <v>10.1.10.0</v>
+      </c>
+      <c r="E5" s="7" t="str">
+        <f>LEFT(D5,LEN(D5)-1)&amp;"1"</f>
+        <v>10.1.10.1</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="G5" s="7" t="str" cm="1">
+        <f t="array" ref="G5">_xlfn.LET(
+_xlpm.net,SUM(--_xlfn.TEXTSPLIT(Tabell6[[#This Row],[nett id]],".")*{16777216,65536,256,1}),
+_xlpm.addr,_xlpm.net+1,
+_xlfn.TEXTJOIN(".",TRUE,MOD(QUOTIENT(_xlpm.addr,{16777216,65536,256,1}),256))
+)</f>
+        <v>10.1.10.1</v>
+      </c>
+      <c r="H5" s="7" t="str" cm="1">
+        <f t="array" ref="H5">_xlfn.LET(
+_xlpm.net,SUM(--_xlfn.TEXTSPLIT(Tabell6[[#This Row],[nett id]],".")*{16777216,65536,256,1}),
+_xlpm.mask,SUM(--_xlfn.TEXTSPLIT(Tabell6[[#This Row],[mask]],".")*{16777216,65536,256,1}),
+_xlpm.addr,_xlpm.net+(4294967295-_xlpm.mask)-1,
+_xlfn.TEXTJOIN(".",TRUE,MOD(QUOTIENT(_xlpm.addr,{16777216,65536,256,1}),256))
+)</f>
+        <v>10.1.10.254</v>
+      </c>
+      <c r="I5" s="7">
+        <v>40</v>
+      </c>
+      <c r="J5" s="9">
+        <v>21</v>
+      </c>
+      <c r="K5" s="9">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="G5" s="8" t="str">
-        <f t="shared" ref="G5:G7" si="1">LEFT(D5,LEN(D5)-1)&amp;"1"</f>
-        <v>10.11.0.1</v>
-      </c>
-      <c r="H5" s="8" t="str">
-        <f>LEFT(D5,FIND(".",D5,FIND(".",D5)+1)-1)&amp;".255.254"</f>
-        <v>10.11.255.254</v>
-      </c>
-      <c r="I5" s="8">
+      <c r="B6" s="8">
+        <v>20</v>
+      </c>
+      <c r="C6" s="7">
+        <v>0</v>
+      </c>
+      <c r="D6" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>10.1.20.0</v>
+      </c>
+      <c r="E6" s="7" t="str">
+        <f t="shared" ref="E5:E7" si="1">LEFT(D6,LEN(D6)-1)&amp;"1"</f>
+        <v>10.1.20.1</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="G6" s="7" t="str" cm="1">
+        <f t="array" ref="G6">_xlfn.LET(
+_xlpm.net,SUM(--_xlfn.TEXTSPLIT(Tabell6[[#This Row],[nett id]],".")*{16777216,65536,256,1}),
+_xlpm.addr,_xlpm.net+1,
+_xlfn.TEXTJOIN(".",TRUE,MOD(QUOTIENT(_xlpm.addr,{16777216,65536,256,1}),256))
+)</f>
+        <v>10.1.20.1</v>
+      </c>
+      <c r="H6" s="7" t="str" cm="1">
+        <f t="array" ref="H6">_xlfn.LET(
+_xlpm.net,SUM(--_xlfn.TEXTSPLIT(Tabell6[[#This Row],[nett id]],".")*{16777216,65536,256,1}),
+_xlpm.mask,SUM(--_xlfn.TEXTSPLIT(Tabell6[[#This Row],[mask]],".")*{16777216,65536,256,1}),
+_xlpm.addr,_xlpm.net+(4294967295-_xlpm.mask)-1,
+_xlfn.TEXTJOIN(".",TRUE,MOD(QUOTIENT(_xlpm.addr,{16777216,65536,256,1}),256))
+)</f>
+        <v>10.1.20.254</v>
+      </c>
+      <c r="I6" s="7">
         <v>40</v>
       </c>
-      <c r="J5" s="10">
-        <v>21</v>
-      </c>
-      <c r="K5" s="10">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="8" t="s">
+      <c r="J6" s="9">
+        <v>11</v>
+      </c>
+      <c r="K6" s="9">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B6" s="9">
-        <v>20</v>
-      </c>
-      <c r="C6" s="8">
+      <c r="B7" s="8">
+        <v>30</v>
+      </c>
+      <c r="C7" s="7">
         <v>0</v>
       </c>
-      <c r="D6" s="8" t="str">
-        <f>10&amp;"."&amp;(B6+A2)&amp;"."&amp;0&amp;"."&amp;0</f>
-        <v>10.21.0.0</v>
-      </c>
-      <c r="E6" s="8" t="str">
+      <c r="D7" s="7" t="str">
         <f t="shared" si="0"/>
-        <v>10.21.0.1</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="G6" s="8" t="str">
+        <v>10.1.30.0</v>
+      </c>
+      <c r="E7" s="7" t="str">
         <f t="shared" si="1"/>
-        <v>10.21.0.1</v>
-      </c>
-      <c r="H6" s="8" t="str">
-        <f>LEFT(D6,FIND(".",D6,FIND(".",D6)+1)-1)&amp;".255.254"</f>
-        <v>10.21.255.254</v>
-      </c>
-      <c r="I6" s="8">
-        <v>40</v>
-      </c>
-      <c r="J6" s="10">
-        <v>11</v>
-      </c>
-      <c r="K6" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="B7" s="9">
-        <v>30</v>
-      </c>
-      <c r="C7" s="8">
-        <v>0</v>
-      </c>
-      <c r="D7" s="8" t="str">
-        <f>10&amp;"."&amp;(B7+A2)&amp;"."&amp;0&amp;"."&amp;0</f>
-        <v>10.31.0.0</v>
-      </c>
-      <c r="E7" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>10.31.0.1</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="G7" s="8" t="str">
-        <f t="shared" si="1"/>
-        <v>10.31.0.1</v>
-      </c>
-      <c r="H7" s="8" t="str">
-        <f>LEFT(D7,FIND(".",D7,FIND(".",D7)+1)-1)&amp;".255.254"</f>
-        <v>10.31.255.254</v>
-      </c>
-      <c r="I7" s="8">
+        <v>10.1.30.1</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="G7" s="7" t="str" cm="1">
+        <f t="array" ref="G7">_xlfn.LET(
+_xlpm.net,SUM(--_xlfn.TEXTSPLIT(Tabell6[[#This Row],[nett id]],".")*{16777216,65536,256,1}),
+_xlpm.addr,_xlpm.net+1,
+_xlfn.TEXTJOIN(".",TRUE,MOD(QUOTIENT(_xlpm.addr,{16777216,65536,256,1}),256))
+)</f>
+        <v>10.1.30.1</v>
+      </c>
+      <c r="H7" s="7" t="str" cm="1">
+        <f t="array" ref="H7">_xlfn.LET(
+_xlpm.net,SUM(--_xlfn.TEXTSPLIT(Tabell6[[#This Row],[nett id]],".")*{16777216,65536,256,1}),
+_xlpm.mask,SUM(--_xlfn.TEXTSPLIT(Tabell6[[#This Row],[mask]],".")*{16777216,65536,256,1}),
+_xlpm.addr,_xlpm.net+(4294967295-_xlpm.mask)-1,
+_xlfn.TEXTJOIN(".",TRUE,MOD(QUOTIENT(_xlpm.addr,{16777216,65536,256,1}),256))
+)</f>
+        <v>10.1.30.254</v>
+      </c>
+      <c r="I7" s="7">
         <v>40</v>
       </c>
       <c r="J7">
@@ -2762,35 +2644,44 @@
       </c>
     </row>
     <row r="8" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="B8" s="9">
+      <c r="A8" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8" s="8">
         <v>40</v>
       </c>
-      <c r="C8" s="8">
+      <c r="C8" s="7">
         <v>0</v>
       </c>
-      <c r="D8" s="8" t="str">
-        <f>10&amp;"."&amp;(B8+A2)&amp;"."&amp;0&amp;"."&amp;0</f>
-        <v>10.41.0.0</v>
-      </c>
-      <c r="E8" s="8" t="str">
+      <c r="D8" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>10.1.40.0</v>
+      </c>
+      <c r="E8" s="7" t="str">
         <f t="shared" ref="E8" si="2">LEFT(D8,LEN(D8)-1)&amp;"1"</f>
-        <v>10.41.0.1</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="G8" s="8" t="str">
-        <f t="shared" ref="G8" si="3">LEFT(D8,LEN(D8)-1)&amp;"1"</f>
-        <v>10.41.0.1</v>
-      </c>
-      <c r="H8" s="8" t="str">
-        <f>LEFT(D8,FIND(".",D8,FIND(".",D8)+1)-1)&amp;".255.254"</f>
-        <v>10.41.255.254</v>
-      </c>
-      <c r="I8" s="8">
+        <v>10.1.40.1</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="G8" s="7" t="str" cm="1">
+        <f t="array" ref="G8">_xlfn.LET(
+_xlpm.net,SUM(--_xlfn.TEXTSPLIT(Tabell6[[#This Row],[nett id]],".")*{16777216,65536,256,1}),
+_xlpm.addr,_xlpm.net+1,
+_xlfn.TEXTJOIN(".",TRUE,MOD(QUOTIENT(_xlpm.addr,{16777216,65536,256,1}),256))
+)</f>
+        <v>10.1.40.1</v>
+      </c>
+      <c r="H8" s="7" t="str" cm="1">
+        <f t="array" ref="H8">_xlfn.LET(
+_xlpm.net,SUM(--_xlfn.TEXTSPLIT(Tabell6[[#This Row],[nett id]],".")*{16777216,65536,256,1}),
+_xlpm.mask,SUM(--_xlfn.TEXTSPLIT(Tabell6[[#This Row],[mask]],".")*{16777216,65536,256,1}),
+_xlpm.addr,_xlpm.net+(4294967295-_xlpm.mask)-1,
+_xlfn.TEXTJOIN(".",TRUE,MOD(QUOTIENT(_xlpm.addr,{16777216,65536,256,1}),256))
+)</f>
+        <v>10.1.40.254</v>
+      </c>
+      <c r="I8" s="7">
         <v>40</v>
       </c>
       <c r="J8">
@@ -2809,126 +2700,126 @@
         <v>19</v>
       </c>
       <c r="B10" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="D10" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="D10" s="6" t="s">
+    </row>
+    <row r="11" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B11" s="17" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="11" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="B11" s="18" t="s">
-        <v>38</v>
-      </c>
-      <c r="C11" s="8">
+      <c r="C11" s="7">
         <v>10</v>
       </c>
-      <c r="D11" s="8" t="str">
+      <c r="D11" s="7" t="str">
         <f>$A$2&amp;"."&amp;$A$2&amp;"."&amp;$A$2&amp;"."&amp;(C11)</f>
         <v>1.1.1.10</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="8" t="s">
+      <c r="A12" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B12" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" s="7">
+        <v>20</v>
+      </c>
+      <c r="D12" s="7" t="str">
+        <f t="shared" ref="D12:D14" si="3">$A$2&amp;"."&amp;$A$2&amp;"."&amp;$A$2&amp;"."&amp;(C12)</f>
+        <v>1.1.1.20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B12" s="18" t="s">
+      <c r="B13" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="C12" s="8">
-        <v>20</v>
-      </c>
-      <c r="D12" s="8" t="str">
-        <f t="shared" ref="D12:D14" si="4">$A$2&amp;"."&amp;$A$2&amp;"."&amp;$A$2&amp;"."&amp;(C12)</f>
-        <v>1.1.1.20</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="8" t="s">
+      <c r="C13" s="7">
+        <v>30</v>
+      </c>
+      <c r="D13" s="7" t="str">
+        <f t="shared" si="3"/>
+        <v>1.1.1.30</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B13" s="18" t="s">
+      <c r="B14" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="C13" s="8">
-        <v>30</v>
-      </c>
-      <c r="D13" s="8" t="str">
-        <f t="shared" si="4"/>
-        <v>1.1.1.30</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="B14" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="C14" s="8">
+      <c r="C14" s="7">
         <v>40</v>
       </c>
-      <c r="D14" s="8" t="str">
-        <f t="shared" si="4"/>
+      <c r="D14" s="7" t="str">
+        <f t="shared" si="3"/>
         <v>1.1.1.40</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="16" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B16" s="6" t="s">
         <v>19</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D16" s="6" t="s">
         <v>24</v>
       </c>
       <c r="E16" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="F16" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="F16" s="6" t="s">
+      <c r="G16" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="G16" s="6" t="s">
+      <c r="H16" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="H16" s="1" t="s">
+      <c r="I16" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="I16" s="1" t="s">
+      <c r="J16" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="J16" s="1" t="s">
+    </row>
+    <row r="17" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="7" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="17" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="8" t="s">
+      <c r="B17" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C17" s="7" t="str">
+        <f t="shared" ref="C17:C19" si="4">172&amp;"."&amp;16&amp;"."&amp;$H17&amp;"."&amp;($A$2)</f>
+        <v>172.16.10.1</v>
+      </c>
+      <c r="D17" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="B17" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="C17" s="8" t="str">
-        <f>172&amp;"."&amp;16&amp;"."&amp;0&amp;"."&amp;(H17+$A$2)</f>
-        <v>172.16.0.11</v>
-      </c>
-      <c r="D17" s="8" t="s">
+      <c r="E17" s="13"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="7" t="s">
         <v>51</v>
-      </c>
-      <c r="E17" s="14"/>
-      <c r="F17" s="8"/>
-      <c r="G17" s="8" t="s">
-        <v>52</v>
       </c>
       <c r="H17" s="2">
         <v>10</v>
@@ -2937,23 +2828,23 @@
       <c r="J17" s="2"/>
     </row>
     <row r="18" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="B18" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="C18" s="8" t="str">
-        <f t="shared" ref="C18" si="5">172&amp;"."&amp;16&amp;"."&amp;0&amp;"."&amp;(H18+$A$2)</f>
-        <v>172.16.0.31</v>
-      </c>
-      <c r="D18" s="8" t="s">
+      <c r="A18" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C18" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>172.16.30.1</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="E18" s="13"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="7" t="s">
         <v>51</v>
-      </c>
-      <c r="E18" s="14"/>
-      <c r="F18" s="8"/>
-      <c r="G18" s="8" t="s">
-        <v>52</v>
       </c>
       <c r="H18" s="2">
         <v>30</v>
@@ -2964,23 +2855,23 @@
       <c r="J18" s="2"/>
     </row>
     <row r="19" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="B19" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="C19" s="8" t="str">
-        <f t="shared" ref="C19" si="6">172&amp;"."&amp;16&amp;"."&amp;0&amp;"."&amp;(H19+$A$2)</f>
-        <v>172.16.0.41</v>
-      </c>
-      <c r="D19" s="8" t="s">
+      <c r="A19" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C19" s="7" t="str">
+        <f t="shared" si="4"/>
+        <v>172.16.40.1</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="E19" s="13"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="7" t="s">
         <v>51</v>
-      </c>
-      <c r="E19" s="14"/>
-      <c r="F19" s="8"/>
-      <c r="G19" s="8" t="s">
-        <v>52</v>
       </c>
       <c r="H19" s="2">
         <v>40</v>
@@ -2991,13 +2882,13 @@
       <c r="J19" s="2"/>
     </row>
     <row r="20" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="12"/>
-      <c r="B20" s="12"/>
-      <c r="C20" s="12"/>
-      <c r="D20" s="12"/>
-      <c r="E20" s="12"/>
-      <c r="F20" s="12"/>
-      <c r="G20" s="12"/>
+      <c r="A20" s="11"/>
+      <c r="B20" s="11"/>
+      <c r="C20" s="11"/>
+      <c r="D20" s="11"/>
+      <c r="E20" s="11"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="11"/>
     </row>
     <row r="21" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
@@ -3016,10 +2907,10 @@
         <v>6</v>
       </c>
       <c r="F21" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G21" s="1" t="s">
         <v>55</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="22" spans="1:12" ht="28.7" customHeight="1" x14ac:dyDescent="0.2">
@@ -3043,80 +2934,80 @@
         <v>2</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="H22" s="19"/>
+        <v>56</v>
+      </c>
+      <c r="H22" s="18"/>
     </row>
     <row r="23" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="24" spans="1:12" ht="39" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="15" t="s">
+      <c r="A24" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="B24" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="B24" s="15" t="s">
+      <c r="C24" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="C24" s="15" t="s">
+      <c r="D24" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="E24" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="F24" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="D24" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="E24" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="F24" s="15" t="s">
+      <c r="G24" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="G24" s="15" t="s">
+      <c r="H24" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="H24" s="15" t="s">
+      <c r="I24" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="I24" s="15" t="s">
+      <c r="J24" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="K24" s="14" t="s">
         <v>64</v>
       </c>
-      <c r="J24" s="15" t="s">
-        <v>1</v>
-      </c>
-      <c r="K24" s="15" t="s">
+      <c r="L24" s="33" t="s">
         <v>65</v>
       </c>
-      <c r="L24" t="s">
-        <v>66</v>
-      </c>
     </row>
     <row r="25" spans="1:12" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="8">
+      <c r="A25" s="7">
         <f>(ROW())-(ROW()-1)</f>
         <v>1</v>
       </c>
-      <c r="B25" s="8">
+      <c r="B25" s="7">
         <v>10</v>
       </c>
-      <c r="C25" s="8" t="str">
+      <c r="C25" s="7" t="str">
         <f>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A25)</f>
-        <v>10.11.0.2</v>
-      </c>
-      <c r="D25" s="8" t="str">
+        <v>10.1.10.2</v>
+      </c>
+      <c r="D25" s="7" t="str">
         <f>$E$5</f>
-        <v>10.11.0.1</v>
-      </c>
-      <c r="E25" s="8" t="str">
+        <v>10.1.10.1</v>
+      </c>
+      <c r="E25" s="7" t="str">
         <f>$F$5</f>
-        <v>255.255.0.0</v>
-      </c>
-      <c r="F25" s="8">
+        <v>255.255.255.0</v>
+      </c>
+      <c r="F25" s="7">
         <v>24</v>
       </c>
-      <c r="G25" s="8">
+      <c r="G25" s="7">
         <v>1</v>
       </c>
-      <c r="H25" s="11">
+      <c r="H25" s="10">
         <v>3</v>
       </c>
-      <c r="I25" s="8" t="s">
-        <v>67</v>
+      <c r="I25" s="7" t="s">
+        <v>66</v>
       </c>
       <c r="J25" s="2" t="s">
         <v>12</v>
@@ -3125,52 +3016,44 @@
         <f>IF($A25=1,F25-G25-H25*$F$22-2-IF($K$2&lt;&gt;$L$2,1,0)-IF(OR(UPPER($G$22)="SPAN",UPPER($G$22)="ERSPAN",UPPER($G$22)="RSPAN"),1,0),F25-G25-(1+H25)*$F$22-1)</f>
         <v>14</v>
       </c>
-      <c r="L25" t="str">
-        <f>10&amp;"."&amp;(50+$A$2)&amp;"."&amp;0&amp;"."&amp;(A25+1)</f>
-        <v>10.51.0.2</v>
-      </c>
     </row>
     <row r="26" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="17">
+      <c r="A26" s="16">
         <v>2</v>
       </c>
-      <c r="B26" s="17">
+      <c r="B26" s="16">
         <v>10</v>
       </c>
-      <c r="C26" s="17" t="str">
+      <c r="C26" s="16" t="str">
         <f>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A26)</f>
-        <v>10.11.0.3</v>
-      </c>
-      <c r="D26" s="17" t="str">
+        <v>10.1.10.3</v>
+      </c>
+      <c r="D26" s="16" t="str">
         <f>$E$5</f>
-        <v>10.11.0.1</v>
-      </c>
-      <c r="E26" s="17" t="str">
+        <v>10.1.10.1</v>
+      </c>
+      <c r="E26" s="16" t="str">
         <f>$F$5</f>
-        <v>255.255.0.0</v>
-      </c>
-      <c r="F26" s="17">
+        <v>255.255.255.0</v>
+      </c>
+      <c r="F26" s="16">
         <v>24</v>
       </c>
-      <c r="G26" s="17">
+      <c r="G26" s="16">
         <v>1</v>
       </c>
-      <c r="H26" s="17">
+      <c r="H26" s="16">
         <v>0</v>
       </c>
-      <c r="I26" s="16" t="s">
-        <v>67</v>
-      </c>
-      <c r="J26" s="13" t="s">
+      <c r="I26" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="J26" s="12" t="s">
         <v>12</v>
       </c>
       <c r="K26" s="2">
         <f>IF($A26=1,F26-G26-H26*$F$22-2-IF($K$2&lt;&gt;$L$2,1,0)-IF(OR(UPPER($G$22)="SPAN",UPPER($G$22)="ERSPAN",UPPER($G$22)="RSPAN"),1,0),F26-G26-(1+H26)*$F$22-1)</f>
         <v>20</v>
-      </c>
-      <c r="L26" t="str">
-        <f>10&amp;"."&amp;(50+$A$2)&amp;"."&amp;0&amp;"."&amp;(A26+1)</f>
-        <v>10.51.0.3</v>
       </c>
     </row>
     <row r="27" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -4177,598 +4060,634 @@
   <dimension ref="A1:M994"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.7109375" style="14" customWidth="1"/>
-    <col min="2" max="2" width="13" style="14" customWidth="1"/>
-    <col min="3" max="3" width="75.85546875" style="14" customWidth="1"/>
-    <col min="4" max="4" width="12.28515625" style="14" customWidth="1"/>
-    <col min="5" max="5" width="75.85546875" style="14" customWidth="1"/>
-    <col min="6" max="6" width="16.85546875" style="14" customWidth="1"/>
-    <col min="7" max="7" width="75.85546875" style="14" customWidth="1"/>
-    <col min="8" max="8" width="22" style="14" customWidth="1"/>
-    <col min="9" max="9" width="25.5703125" style="14" customWidth="1"/>
-    <col min="10" max="10" width="11.28515625" style="14" customWidth="1"/>
-    <col min="11" max="11" width="18" style="14" customWidth="1"/>
+    <col min="1" max="1" width="10.7109375" style="13" customWidth="1"/>
+    <col min="2" max="2" width="13" style="13" customWidth="1"/>
+    <col min="3" max="3" width="75.85546875" style="13" customWidth="1"/>
+    <col min="4" max="4" width="12.28515625" style="13" customWidth="1"/>
+    <col min="5" max="5" width="75.85546875" style="13" customWidth="1"/>
+    <col min="6" max="6" width="16.85546875" style="13" customWidth="1"/>
+    <col min="7" max="7" width="75.85546875" style="13" customWidth="1"/>
+    <col min="8" max="8" width="22" style="13" customWidth="1"/>
+    <col min="9" max="9" width="25.5703125" style="13" customWidth="1"/>
+    <col min="10" max="10" width="11.28515625" style="13" customWidth="1"/>
+    <col min="11" max="11" width="18" style="13" customWidth="1"/>
     <col min="12" max="12" width="18" customWidth="1"/>
     <col min="13" max="13" width="14" customWidth="1"/>
-    <col min="14" max="16384" width="12.5703125" style="14"/>
+    <col min="14" max="16384" width="12.5703125" style="13"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="C1" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="14" t="s">
+      <c r="E1" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="14" t="s">
+      <c r="F1" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="14" t="s">
+      <c r="G1" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="14" t="s">
+      <c r="H1" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="14" t="s">
+      <c r="I1" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="31" t="s">
+      <c r="J1" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="K1" s="31" t="s">
+      <c r="K1" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="L1" s="32" t="s">
-        <v>68</v>
+      <c r="L1" s="31" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="14">
+      <c r="A2" s="13">
         <v>2</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="14" t="str">
+      <c r="C2" s="13" t="str">
         <f>A2&amp;"."&amp;A2&amp;"."&amp;A2&amp;".0"</f>
         <v>2.2.2.0</v>
       </c>
-      <c r="D2" s="14" t="s">
+      <c r="D2" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="14" t="s">
+      <c r="E2" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="F2" s="14" t="s">
+      <c r="F2" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="G2" s="14" t="s">
+      <c r="G2" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="H2" s="14" t="str">
+      <c r="H2" s="13" t="str">
         <f>'Site 1 (HUB)'!H2</f>
         <v>TACACS-KEY</v>
       </c>
-      <c r="I2" s="14" t="s">
+      <c r="I2" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="J2" s="23" t="str">
+      <c r="J2" s="22" t="str">
         <f>'Site 1 (HUB)'!K2</f>
         <v>10.11.0.10</v>
       </c>
-      <c r="K2" s="23" t="str">
+      <c r="K2" s="22" t="str">
         <f>'Site 1 (HUB)'!L2</f>
         <v>10.11.0.10</v>
       </c>
-      <c r="L2" s="23" t="str">
+      <c r="L2" s="22" t="str">
         <f>'Site 1 (HUB)'!M2</f>
         <v>OFF</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="1:12" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="B4" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="C4" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="D4" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="14" t="s">
+      <c r="E4" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="F4" s="14" t="s">
+      <c r="F4" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="G4" s="14" t="s">
+      <c r="G4" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="H4" s="14" t="s">
+      <c r="H4" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="I4" s="14" t="s">
+      <c r="I4" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="J4" s="14" t="s">
+      <c r="J4" s="32" t="s">
         <v>28</v>
       </c>
-      <c r="K4" s="14" t="s">
+      <c r="K4" s="32" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B5" s="14">
+      <c r="B5" s="8">
         <v>10</v>
       </c>
-      <c r="C5" s="14">
+      <c r="C5" s="7">
         <v>0</v>
       </c>
-      <c r="D5" s="14" t="str">
-        <f>10&amp;"."&amp;(B5+A2)&amp;"."&amp;0&amp;"."&amp;0</f>
-        <v>10.12.0.0</v>
-      </c>
-      <c r="E5" s="14" t="str">
-        <f t="shared" ref="E5:E8" si="0">LEFT(D5,LEN(D5)-1)&amp;"1"</f>
-        <v>10.12.0.1</v>
-      </c>
-      <c r="F5" s="14" t="s">
+      <c r="D5" s="7" t="str">
+        <f t="shared" ref="D5:D8" si="0">10&amp;"."&amp;($A$2)&amp;"."&amp;$B5&amp;"."&amp;0</f>
+        <v>10.2.10.0</v>
+      </c>
+      <c r="E5" s="7" t="str">
+        <f>LEFT(D5,LEN(D5)-1)&amp;"1"</f>
+        <v>10.2.10.1</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="G5" s="7" t="str" cm="1">
+        <f t="array" ref="G5">_xlfn.LET(
+_xlpm.net,SUM(--_xlfn.TEXTSPLIT(Tabell62[[#This Row],[nett id]],".")*{16777216,65536,256,1}),
+_xlpm.addr,_xlpm.net+1,
+_xlfn.TEXTJOIN(".",TRUE,MOD(QUOTIENT(_xlpm.addr,{16777216,65536,256,1}),256))
+)</f>
+        <v>10.2.10.1</v>
+      </c>
+      <c r="H5" s="7" t="str" cm="1">
+        <f t="array" ref="H5">_xlfn.LET(
+_xlpm.net,SUM(--_xlfn.TEXTSPLIT(Tabell62[[#This Row],[nett id]],".")*{16777216,65536,256,1}),
+_xlpm.mask,SUM(--_xlfn.TEXTSPLIT(Tabell62[[#This Row],[mask]],".")*{16777216,65536,256,1}),
+_xlpm.addr,_xlpm.net+(4294967295-_xlpm.mask)-1,
+_xlfn.TEXTJOIN(".",TRUE,MOD(QUOTIENT(_xlpm.addr,{16777216,65536,256,1}),256))
+)</f>
+        <v>10.2.10.254</v>
+      </c>
+      <c r="I5" s="7">
+        <v>40</v>
+      </c>
+      <c r="J5" s="9">
+        <v>21</v>
+      </c>
+      <c r="K5" s="9">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="G5" s="14" t="str">
-        <f t="shared" ref="G5:G8" si="1">LEFT(D5,LEN(D5)-1)&amp;"1"</f>
-        <v>10.12.0.1</v>
-      </c>
-      <c r="H5" s="14" t="str">
-        <f>LEFT(D5,FIND(".",D5,FIND(".",D5)+1)-1)&amp;".255.254"</f>
-        <v>10.12.255.254</v>
-      </c>
-      <c r="I5" s="14">
+      <c r="B6" s="8">
+        <v>20</v>
+      </c>
+      <c r="C6" s="7">
+        <v>0</v>
+      </c>
+      <c r="D6" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>10.2.20.0</v>
+      </c>
+      <c r="E6" s="7" t="str">
+        <f t="shared" ref="E6:E8" si="1">LEFT(D6,LEN(D6)-1)&amp;"1"</f>
+        <v>10.2.20.1</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="G6" s="7" t="str" cm="1">
+        <f t="array" ref="G6">_xlfn.LET(
+_xlpm.net,SUM(--_xlfn.TEXTSPLIT(Tabell62[[#This Row],[nett id]],".")*{16777216,65536,256,1}),
+_xlpm.addr,_xlpm.net+1,
+_xlfn.TEXTJOIN(".",TRUE,MOD(QUOTIENT(_xlpm.addr,{16777216,65536,256,1}),256))
+)</f>
+        <v>10.2.20.1</v>
+      </c>
+      <c r="H6" s="7" t="str" cm="1">
+        <f t="array" ref="H6">_xlfn.LET(
+_xlpm.net,SUM(--_xlfn.TEXTSPLIT(Tabell62[[#This Row],[nett id]],".")*{16777216,65536,256,1}),
+_xlpm.mask,SUM(--_xlfn.TEXTSPLIT(Tabell62[[#This Row],[mask]],".")*{16777216,65536,256,1}),
+_xlpm.addr,_xlpm.net+(4294967295-_xlpm.mask)-1,
+_xlfn.TEXTJOIN(".",TRUE,MOD(QUOTIENT(_xlpm.addr,{16777216,65536,256,1}),256))
+)</f>
+        <v>10.2.20.254</v>
+      </c>
+      <c r="I6" s="7">
         <v>40</v>
       </c>
-      <c r="J5" s="14">
-        <v>21</v>
-      </c>
-      <c r="K5" s="14">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="14" t="s">
+      <c r="J6" s="9">
+        <v>11</v>
+      </c>
+      <c r="K6" s="9">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B6" s="14">
-        <v>20</v>
-      </c>
-      <c r="C6" s="14">
+      <c r="B7" s="8">
+        <v>30</v>
+      </c>
+      <c r="C7" s="7">
         <v>0</v>
       </c>
-      <c r="D6" s="14" t="str">
-        <f>10&amp;"."&amp;(B6+A2)&amp;"."&amp;0&amp;"."&amp;0</f>
-        <v>10.22.0.0</v>
-      </c>
-      <c r="E6" s="14" t="str">
+      <c r="D7" s="7" t="str">
         <f t="shared" si="0"/>
-        <v>10.22.0.1</v>
-      </c>
-      <c r="F6" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="G6" s="14" t="str">
+        <v>10.2.30.0</v>
+      </c>
+      <c r="E7" s="7" t="str">
         <f t="shared" si="1"/>
-        <v>10.22.0.1</v>
-      </c>
-      <c r="H6" s="14" t="str">
-        <f>LEFT(D6,FIND(".",D6,FIND(".",D6)+1)-1)&amp;".255.254"</f>
-        <v>10.22.255.254</v>
-      </c>
-      <c r="I6" s="14">
+        <v>10.2.30.1</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="G7" s="7" t="str" cm="1">
+        <f t="array" ref="G7">_xlfn.LET(
+_xlpm.net,SUM(--_xlfn.TEXTSPLIT(Tabell62[[#This Row],[nett id]],".")*{16777216,65536,256,1}),
+_xlpm.addr,_xlpm.net+1,
+_xlfn.TEXTJOIN(".",TRUE,MOD(QUOTIENT(_xlpm.addr,{16777216,65536,256,1}),256))
+)</f>
+        <v>10.2.30.1</v>
+      </c>
+      <c r="H7" s="7" t="str" cm="1">
+        <f t="array" ref="H7">_xlfn.LET(
+_xlpm.net,SUM(--_xlfn.TEXTSPLIT(Tabell62[[#This Row],[nett id]],".")*{16777216,65536,256,1}),
+_xlpm.mask,SUM(--_xlfn.TEXTSPLIT(Tabell62[[#This Row],[mask]],".")*{16777216,65536,256,1}),
+_xlpm.addr,_xlpm.net+(4294967295-_xlpm.mask)-1,
+_xlfn.TEXTJOIN(".",TRUE,MOD(QUOTIENT(_xlpm.addr,{16777216,65536,256,1}),256))
+)</f>
+        <v>10.2.30.254</v>
+      </c>
+      <c r="I7" s="7">
         <v>40</v>
       </c>
-      <c r="J6" s="14">
-        <v>11</v>
-      </c>
-      <c r="K6" s="14">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="14" t="s">
+      <c r="J7">
+        <v>42</v>
+      </c>
+      <c r="K7">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B7" s="14">
-        <v>30</v>
-      </c>
-      <c r="C7" s="14">
+      <c r="B8" s="8">
+        <v>40</v>
+      </c>
+      <c r="C8" s="7">
         <v>0</v>
       </c>
-      <c r="D7" s="14" t="str">
-        <f>10&amp;"."&amp;(B7+A2)&amp;"."&amp;0&amp;"."&amp;0</f>
-        <v>10.32.0.0</v>
-      </c>
-      <c r="E7" s="14" t="str">
+      <c r="D8" s="7" t="str">
         <f t="shared" si="0"/>
-        <v>10.32.0.1</v>
-      </c>
-      <c r="F7" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="G7" s="14" t="str">
+        <v>10.2.40.0</v>
+      </c>
+      <c r="E8" s="7" t="str">
         <f t="shared" si="1"/>
-        <v>10.32.0.1</v>
-      </c>
-      <c r="H7" s="14" t="str">
-        <f>LEFT(D7,FIND(".",D7,FIND(".",D7)+1)-1)&amp;".255.254"</f>
-        <v>10.32.255.254</v>
-      </c>
-      <c r="I7" s="14">
+        <v>10.2.40.1</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="G8" s="7" t="str" cm="1">
+        <f t="array" ref="G8">_xlfn.LET(
+_xlpm.net,SUM(--_xlfn.TEXTSPLIT(Tabell62[[#This Row],[nett id]],".")*{16777216,65536,256,1}),
+_xlpm.addr,_xlpm.net+1,
+_xlfn.TEXTJOIN(".",TRUE,MOD(QUOTIENT(_xlpm.addr,{16777216,65536,256,1}),256))
+)</f>
+        <v>10.2.40.1</v>
+      </c>
+      <c r="H8" s="7" t="str" cm="1">
+        <f t="array" ref="H8">_xlfn.LET(
+_xlpm.net,SUM(--_xlfn.TEXTSPLIT(Tabell62[[#This Row],[nett id]],".")*{16777216,65536,256,1}),
+_xlpm.mask,SUM(--_xlfn.TEXTSPLIT(Tabell62[[#This Row],[mask]],".")*{16777216,65536,256,1}),
+_xlpm.addr,_xlpm.net+(4294967295-_xlpm.mask)-1,
+_xlfn.TEXTJOIN(".",TRUE,MOD(QUOTIENT(_xlpm.addr,{16777216,65536,256,1}),256))
+)</f>
+        <v>10.2.40.254</v>
+      </c>
+      <c r="I8" s="7">
         <v>40</v>
       </c>
-      <c r="J7" s="14">
-        <v>42</v>
-      </c>
-      <c r="K7" s="14">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="B8" s="14">
-        <v>40</v>
-      </c>
-      <c r="C8" s="14">
-        <v>0</v>
-      </c>
-      <c r="D8" s="14" t="str">
-        <f>10&amp;"."&amp;(B8+A2)&amp;"."&amp;0&amp;"."&amp;0</f>
-        <v>10.42.0.0</v>
-      </c>
-      <c r="E8" s="14" t="str">
-        <f t="shared" si="0"/>
-        <v>10.42.0.1</v>
-      </c>
-      <c r="F8" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="G8" s="14" t="str">
-        <f t="shared" si="1"/>
-        <v>10.42.0.1</v>
-      </c>
-      <c r="H8" s="14" t="str">
-        <f>LEFT(D8,FIND(".",D8,FIND(".",D8)+1)-1)&amp;".255.254"</f>
-        <v>10.42.255.254</v>
-      </c>
-      <c r="I8" s="14">
-        <v>40</v>
-      </c>
-      <c r="J8" s="14">
+      <c r="J8">
         <v>41</v>
       </c>
-      <c r="K8" s="14">
+      <c r="K8">
         <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="10" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="14" t="s">
+      <c r="A10" s="13" t="s">
         <v>19</v>
       </c>
       <c r="B10" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="C10" s="14" t="s">
+      <c r="D10" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="D10" s="14" t="s">
+    </row>
+    <row r="11" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="B11" s="17" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="11" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="B11" s="18" t="s">
-        <v>38</v>
-      </c>
-      <c r="C11" s="14">
+      <c r="C11" s="13">
         <v>10</v>
       </c>
-      <c r="D11" s="14" t="str">
+      <c r="D11" s="13" t="str">
         <f>A2&amp;"."&amp;A2&amp;"."&amp;A2&amp;"."&amp;(C11)</f>
         <v>2.2.2.10</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="B12" s="18" t="s">
-        <v>39</v>
-      </c>
-      <c r="C12" s="14">
+      <c r="A12" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="B12" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" s="13">
         <v>20</v>
       </c>
-      <c r="D12" s="14" t="str">
+      <c r="D12" s="13" t="str">
         <f>A2&amp;"."&amp;A2&amp;"."&amp;A2&amp;"."&amp;(C12)</f>
         <v>2.2.2.20</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="B13" s="18" t="s">
-        <v>40</v>
-      </c>
-      <c r="C13" s="14">
+      <c r="A13" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="B13" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="C13" s="13">
         <v>30</v>
       </c>
-      <c r="D13" s="14" t="str">
+      <c r="D13" s="13" t="str">
         <f>A2&amp;"."&amp;A2&amp;"."&amp;A2&amp;"."&amp;(C13)</f>
         <v>2.2.2.30</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="B14" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="C14" s="14">
+      <c r="A14" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="B14" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="D14" s="14" t="str">
+      <c r="C14" s="13">
+        <v>40</v>
+      </c>
+      <c r="D14" s="13" t="str">
         <f t="shared" ref="D14" si="2">$A$2&amp;"."&amp;$A$2&amp;"."&amp;$A$2&amp;"."&amp;(C14)</f>
         <v>2.2.2.40</v>
       </c>
     </row>
     <row r="15" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="16" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="14" t="s">
+      <c r="A16" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="B16" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="C16" s="14" t="s">
+      <c r="D16" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="E16" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="D16" s="14" t="s">
-        <v>24</v>
-      </c>
-      <c r="E16" s="14" t="s">
+      <c r="F16" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="F16" s="14" t="s">
+      <c r="G16" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="G16" s="14" t="s">
+      <c r="H16" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="H16" s="14" t="s">
+      <c r="I16" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="I16" s="14" t="s">
+      <c r="J16" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="J16" s="14" t="s">
+    </row>
+    <row r="17" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="13" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="17" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="14" t="s">
-        <v>50</v>
-      </c>
-      <c r="B17" s="14" t="s">
+      <c r="B17" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="C17" s="14" t="str">
+      <c r="C17" s="13" t="str">
         <f>172&amp;"."&amp;16&amp;"."&amp;0&amp;"."&amp;(H17+$A$2)</f>
         <v>172.16.0.12</v>
       </c>
-      <c r="D17" s="14" t="s">
+      <c r="D17" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="G17" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="G17" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="H17" s="14">
+      <c r="H17" s="13">
         <v>10</v>
       </c>
-      <c r="I17" s="14">
+      <c r="I17" s="13">
         <f t="array" ref="I17">'Site 1 (HUB)'!I17</f>
         <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="B18" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="C18" s="14" t="str">
+      <c r="A18" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="C18" s="13" t="str">
         <f>172&amp;"."&amp;16&amp;"."&amp;0&amp;"."&amp;(H18+$A$2)</f>
         <v>172.16.0.32</v>
       </c>
-      <c r="D18" s="14" t="s">
+      <c r="D18" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="G18" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="G18" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="H18" s="14">
+      <c r="H18" s="13">
         <v>30</v>
       </c>
-      <c r="I18" s="14" t="b">
+      <c r="I18" s="13" t="b">
         <f t="array" ref="I18">'Site 1 (HUB)'!I18</f>
         <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="B19" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="C19" s="14" t="str">
+      <c r="A19" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="C19" s="13" t="str">
         <f t="shared" ref="C19" si="3">172&amp;"."&amp;16&amp;"."&amp;0&amp;"."&amp;(H19+$A$2)</f>
         <v>172.16.0.42</v>
       </c>
-      <c r="D19" s="14" t="s">
+      <c r="D19" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="G19" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="G19" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="H19" s="14">
+      <c r="H19" s="13">
         <v>40</v>
       </c>
-      <c r="I19" s="14" t="b">
+      <c r="I19" s="13" t="b">
         <f>'Site 1 (HUB)'!I19</f>
         <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="21" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="14" t="s">
+      <c r="A21" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B21" s="14" t="s">
+      <c r="B21" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="C21" s="14" t="s">
+      <c r="C21" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="D21" s="14" t="s">
+      <c r="D21" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="E21" s="14" t="s">
+      <c r="E21" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="F21" s="14" t="s">
+      <c r="F21" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="G21" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="G21" s="1" t="s">
-        <v>56</v>
-      </c>
       <c r="H21"/>
     </row>
     <row r="22" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="14">
+      <c r="A22" s="13">
         <f>A2</f>
         <v>2</v>
       </c>
-      <c r="B22" s="14" t="s">
+      <c r="B22" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="C22" s="14" t="s">
+      <c r="C22" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="D22" s="14" t="s">
+      <c r="D22" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="E22" s="14" t="s">
+      <c r="E22" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="F22" s="14">
+      <c r="F22" s="13">
         <v>2</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="H22" s="20"/>
+        <v>56</v>
+      </c>
+      <c r="H22" s="19"/>
     </row>
     <row r="23" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="24" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="15" t="s">
+      <c r="A24" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="B24" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="B24" s="15" t="s">
+      <c r="C24" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="C24" s="15" t="s">
+      <c r="D24" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="E24" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="F24" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="D24" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="E24" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="F24" s="15" t="s">
+      <c r="G24" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="G24" s="15" t="s">
+      <c r="H24" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="H24" s="15" t="s">
+      <c r="I24" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="I24" s="15" t="s">
+      <c r="J24" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="K24" s="14" t="s">
         <v>64</v>
       </c>
-      <c r="J24" s="15" t="s">
-        <v>1</v>
-      </c>
-      <c r="K24" s="15" t="s">
+      <c r="L24" t="s">
         <v>65</v>
       </c>
-      <c r="L24" t="s">
-        <v>66</v>
-      </c>
     </row>
     <row r="25" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="8">
+      <c r="A25" s="7">
         <f>(ROW())-(ROW()-1)</f>
         <v>1</v>
       </c>
-      <c r="B25" s="8">
+      <c r="B25" s="7">
         <v>10</v>
       </c>
-      <c r="C25" s="8" t="str">
+      <c r="C25" s="7" t="str">
         <f>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A25)</f>
-        <v>10.12.0.2</v>
-      </c>
-      <c r="D25" s="8" t="str">
+        <v>10.2.10.2</v>
+      </c>
+      <c r="D25" s="7" t="str">
         <f>$E$5</f>
-        <v>10.12.0.1</v>
-      </c>
-      <c r="E25" s="8" t="str">
+        <v>10.2.10.1</v>
+      </c>
+      <c r="E25" s="7" t="str">
         <f>$F$5</f>
-        <v>255.255.0.0</v>
-      </c>
-      <c r="F25" s="8">
+        <v>255.255.255.0</v>
+      </c>
+      <c r="F25" s="7">
         <v>24</v>
       </c>
-      <c r="G25" s="8">
+      <c r="G25" s="7">
         <v>1</v>
       </c>
-      <c r="H25" s="11">
+      <c r="H25" s="10">
         <v>0</v>
       </c>
-      <c r="I25" s="8" t="s">
-        <v>67</v>
+      <c r="I25" s="7" t="s">
+        <v>66</v>
       </c>
       <c r="J25" s="2" t="s">
         <v>12</v>
@@ -5792,699 +5711,735 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="15" x14ac:dyDescent="0.2">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="C1" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="14" t="s">
+      <c r="E1" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="14" t="s">
+      <c r="F1" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="14" t="s">
+      <c r="G1" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="14" t="s">
+      <c r="H1" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="14" t="s">
+      <c r="I1" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="22" t="s">
+      <c r="J1" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="K1" s="31" t="s">
+      <c r="K1" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="L1" s="32" t="s">
-        <v>68</v>
+      <c r="L1" s="31" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A2" s="14">
+      <c r="A2" s="13">
         <v>3</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="14" t="str">
+      <c r="C2" s="13" t="str">
         <f>A2&amp;"."&amp;A2&amp;"."&amp;A2&amp;".0"</f>
         <v>3.3.3.0</v>
       </c>
-      <c r="D2" s="14" t="s">
+      <c r="D2" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="14" t="s">
+      <c r="E2" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="F2" s="14" t="s">
+      <c r="F2" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="G2" s="14" t="s">
+      <c r="G2" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="H2" s="14" t="str">
+      <c r="H2" s="13" t="str">
         <f>'Site 1 (HUB)'!H2</f>
         <v>TACACS-KEY</v>
       </c>
-      <c r="I2" s="14" t="s">
+      <c r="I2" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="J2" s="24" t="str">
+      <c r="J2" s="23" t="str">
         <f>'Site 1 (HUB)'!K2</f>
         <v>10.11.0.10</v>
       </c>
-      <c r="K2" s="23" t="str">
+      <c r="K2" s="22" t="str">
         <f>'Site 1 (HUB)'!L2</f>
         <v>10.11.0.10</v>
       </c>
-      <c r="L2" s="29" t="s">
-        <v>69</v>
+      <c r="L2" s="28" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A3" s="14"/>
-      <c r="B3" s="14"/>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14"/>
-    </row>
-    <row r="4" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A4" s="14" t="s">
+      <c r="A3" s="13"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
+      <c r="H3" s="13"/>
+      <c r="I3" s="13"/>
+      <c r="J3" s="13"/>
+      <c r="K3" s="13"/>
+    </row>
+    <row r="4" spans="1:12" ht="15" x14ac:dyDescent="0.2">
+      <c r="A4" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="B4" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="C4" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="D4" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="14" t="s">
+      <c r="E4" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="F4" s="14" t="s">
+      <c r="F4" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="G4" s="14" t="s">
+      <c r="G4" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="H4" s="14" t="s">
+      <c r="H4" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="I4" s="14" t="s">
+      <c r="I4" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="J4" s="14" t="s">
+      <c r="J4" s="32" t="s">
         <v>28</v>
       </c>
-      <c r="K4" s="14" t="s">
+      <c r="K4" s="32" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B5" s="14">
+      <c r="B5" s="8">
         <v>10</v>
       </c>
-      <c r="C5" s="14">
+      <c r="C5" s="7">
         <v>0</v>
       </c>
-      <c r="D5" s="14" t="str">
-        <f>10&amp;"."&amp;(B5+A2)&amp;"."&amp;0&amp;"."&amp;0</f>
-        <v>10.13.0.0</v>
-      </c>
-      <c r="E5" s="14" t="str">
-        <f t="shared" ref="E5:E8" si="0">LEFT(D5,LEN(D5)-1)&amp;"1"</f>
-        <v>10.13.0.1</v>
-      </c>
-      <c r="F5" s="14" t="s">
+      <c r="D5" s="7" t="str">
+        <f t="shared" ref="D5:D8" si="0">10&amp;"."&amp;($A$2)&amp;"."&amp;$B5&amp;"."&amp;0</f>
+        <v>10.3.10.0</v>
+      </c>
+      <c r="E5" s="7" t="str">
+        <f>LEFT(D5,LEN(D5)-1)&amp;"1"</f>
+        <v>10.3.10.1</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="G5" s="7" t="str" cm="1">
+        <f t="array" ref="G5">_xlfn.LET(
+_xlpm.net,SUM(--_xlfn.TEXTSPLIT(Tabell628[[#This Row],[nett id]],".")*{16777216,65536,256,1}),
+_xlpm.addr,_xlpm.net+1,
+_xlfn.TEXTJOIN(".",TRUE,MOD(QUOTIENT(_xlpm.addr,{16777216,65536,256,1}),256))
+)</f>
+        <v>10.3.10.1</v>
+      </c>
+      <c r="H5" s="7" t="str" cm="1">
+        <f t="array" ref="H5">_xlfn.LET(
+_xlpm.net,SUM(--_xlfn.TEXTSPLIT(Tabell628[[#This Row],[nett id]],".")*{16777216,65536,256,1}),
+_xlpm.mask,SUM(--_xlfn.TEXTSPLIT(Tabell628[[#This Row],[mask]],".")*{16777216,65536,256,1}),
+_xlpm.addr,_xlpm.net+(4294967295-_xlpm.mask)-1,
+_xlfn.TEXTJOIN(".",TRUE,MOD(QUOTIENT(_xlpm.addr,{16777216,65536,256,1}),256))
+)</f>
+        <v>10.3.10.254</v>
+      </c>
+      <c r="I5" s="7">
+        <v>40</v>
+      </c>
+      <c r="J5" s="9">
+        <v>21</v>
+      </c>
+      <c r="K5" s="9">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A6" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="G5" s="14" t="str">
-        <f t="shared" ref="G5:G8" si="1">LEFT(D5,LEN(D5)-1)&amp;"1"</f>
-        <v>10.13.0.1</v>
-      </c>
-      <c r="H5" s="14" t="str">
-        <f>LEFT(D5,FIND(".",D5,FIND(".",D5)+1)-1)&amp;".255.254"</f>
-        <v>10.13.255.254</v>
-      </c>
-      <c r="I5" s="14">
+      <c r="B6" s="8">
+        <v>20</v>
+      </c>
+      <c r="C6" s="7">
+        <v>0</v>
+      </c>
+      <c r="D6" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>10.3.20.0</v>
+      </c>
+      <c r="E6" s="7" t="str">
+        <f t="shared" ref="E6:E8" si="1">LEFT(D6,LEN(D6)-1)&amp;"1"</f>
+        <v>10.3.20.1</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="G6" s="7" t="str" cm="1">
+        <f t="array" ref="G6">_xlfn.LET(
+_xlpm.net,SUM(--_xlfn.TEXTSPLIT(Tabell628[[#This Row],[nett id]],".")*{16777216,65536,256,1}),
+_xlpm.addr,_xlpm.net+1,
+_xlfn.TEXTJOIN(".",TRUE,MOD(QUOTIENT(_xlpm.addr,{16777216,65536,256,1}),256))
+)</f>
+        <v>10.3.20.1</v>
+      </c>
+      <c r="H6" s="7" t="str" cm="1">
+        <f t="array" ref="H6">_xlfn.LET(
+_xlpm.net,SUM(--_xlfn.TEXTSPLIT(Tabell628[[#This Row],[nett id]],".")*{16777216,65536,256,1}),
+_xlpm.mask,SUM(--_xlfn.TEXTSPLIT(Tabell628[[#This Row],[mask]],".")*{16777216,65536,256,1}),
+_xlpm.addr,_xlpm.net+(4294967295-_xlpm.mask)-1,
+_xlfn.TEXTJOIN(".",TRUE,MOD(QUOTIENT(_xlpm.addr,{16777216,65536,256,1}),256))
+)</f>
+        <v>10.3.20.254</v>
+      </c>
+      <c r="I6" s="7">
         <v>40</v>
       </c>
-      <c r="J5" s="14">
-        <v>21</v>
-      </c>
-      <c r="K5" s="14">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A6" s="14" t="s">
+      <c r="J6" s="9">
+        <v>11</v>
+      </c>
+      <c r="K6" s="9">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A7" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B6" s="14">
-        <v>20</v>
-      </c>
-      <c r="C6" s="14">
+      <c r="B7" s="8">
+        <v>30</v>
+      </c>
+      <c r="C7" s="7">
         <v>0</v>
       </c>
-      <c r="D6" s="14" t="str">
-        <f>10&amp;"."&amp;(B6+A2)&amp;"."&amp;0&amp;"."&amp;0</f>
-        <v>10.23.0.0</v>
-      </c>
-      <c r="E6" s="14" t="str">
+      <c r="D7" s="7" t="str">
         <f t="shared" si="0"/>
-        <v>10.23.0.1</v>
-      </c>
-      <c r="F6" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="G6" s="14" t="str">
+        <v>10.3.30.0</v>
+      </c>
+      <c r="E7" s="7" t="str">
         <f t="shared" si="1"/>
-        <v>10.23.0.1</v>
-      </c>
-      <c r="H6" s="14" t="str">
-        <f>LEFT(D6,FIND(".",D6,FIND(".",D6)+1)-1)&amp;".255.254"</f>
-        <v>10.23.255.254</v>
-      </c>
-      <c r="I6" s="14">
+        <v>10.3.30.1</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="G7" s="7" t="str" cm="1">
+        <f t="array" ref="G7">_xlfn.LET(
+_xlpm.net,SUM(--_xlfn.TEXTSPLIT(Tabell628[[#This Row],[nett id]],".")*{16777216,65536,256,1}),
+_xlpm.addr,_xlpm.net+1,
+_xlfn.TEXTJOIN(".",TRUE,MOD(QUOTIENT(_xlpm.addr,{16777216,65536,256,1}),256))
+)</f>
+        <v>10.3.30.1</v>
+      </c>
+      <c r="H7" s="7" t="str" cm="1">
+        <f t="array" ref="H7">_xlfn.LET(
+_xlpm.net,SUM(--_xlfn.TEXTSPLIT(Tabell628[[#This Row],[nett id]],".")*{16777216,65536,256,1}),
+_xlpm.mask,SUM(--_xlfn.TEXTSPLIT(Tabell628[[#This Row],[mask]],".")*{16777216,65536,256,1}),
+_xlpm.addr,_xlpm.net+(4294967295-_xlpm.mask)-1,
+_xlfn.TEXTJOIN(".",TRUE,MOD(QUOTIENT(_xlpm.addr,{16777216,65536,256,1}),256))
+)</f>
+        <v>10.3.30.254</v>
+      </c>
+      <c r="I7" s="7">
         <v>40</v>
       </c>
-      <c r="J6" s="14">
-        <v>11</v>
-      </c>
-      <c r="K6" s="14">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A7" s="14" t="s">
+      <c r="J7">
+        <v>42</v>
+      </c>
+      <c r="K7">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A8" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B7" s="14">
+      <c r="B8" s="8">
+        <v>40</v>
+      </c>
+      <c r="C8" s="7">
+        <v>0</v>
+      </c>
+      <c r="D8" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>10.3.40.0</v>
+      </c>
+      <c r="E8" s="7" t="str">
+        <f t="shared" si="1"/>
+        <v>10.3.40.1</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="G8" s="7" t="str" cm="1">
+        <f t="array" ref="G8">_xlfn.LET(
+_xlpm.net,SUM(--_xlfn.TEXTSPLIT(Tabell628[[#This Row],[nett id]],".")*{16777216,65536,256,1}),
+_xlpm.addr,_xlpm.net+1,
+_xlfn.TEXTJOIN(".",TRUE,MOD(QUOTIENT(_xlpm.addr,{16777216,65536,256,1}),256))
+)</f>
+        <v>10.3.40.1</v>
+      </c>
+      <c r="H8" s="7" t="str" cm="1">
+        <f t="array" ref="H8">_xlfn.LET(
+_xlpm.net,SUM(--_xlfn.TEXTSPLIT(Tabell628[[#This Row],[nett id]],".")*{16777216,65536,256,1}),
+_xlpm.mask,SUM(--_xlfn.TEXTSPLIT(Tabell628[[#This Row],[mask]],".")*{16777216,65536,256,1}),
+_xlpm.addr,_xlpm.net+(4294967295-_xlpm.mask)-1,
+_xlfn.TEXTJOIN(".",TRUE,MOD(QUOTIENT(_xlpm.addr,{16777216,65536,256,1}),256))
+)</f>
+        <v>10.3.40.254</v>
+      </c>
+      <c r="I8" s="7">
+        <v>40</v>
+      </c>
+      <c r="J8">
+        <v>41</v>
+      </c>
+      <c r="K8">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A9" s="13"/>
+      <c r="B9" s="13"/>
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="13"/>
+      <c r="F9" s="13"/>
+      <c r="G9" s="13"/>
+      <c r="H9" s="13"/>
+      <c r="I9" s="13"/>
+      <c r="J9" s="13"/>
+      <c r="K9" s="13"/>
+    </row>
+    <row r="10" spans="1:12" ht="15" x14ac:dyDescent="0.2">
+      <c r="A10" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="D10" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="E10" s="13"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="13"/>
+      <c r="H10" s="13"/>
+      <c r="I10" s="13"/>
+      <c r="J10" s="13"/>
+      <c r="K10" s="13"/>
+      <c r="L10" s="13"/>
+    </row>
+    <row r="11" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A11" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="14">
-        <v>0</v>
-      </c>
-      <c r="D7" s="14" t="str">
-        <f>10&amp;"."&amp;(B7+A2)&amp;"."&amp;0&amp;"."&amp;0</f>
-        <v>10.33.0.0</v>
-      </c>
-      <c r="E7" s="14" t="str">
-        <f t="shared" si="0"/>
-        <v>10.33.0.1</v>
-      </c>
-      <c r="F7" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="G7" s="14" t="str">
-        <f t="shared" si="1"/>
-        <v>10.33.0.1</v>
-      </c>
-      <c r="H7" s="14" t="str">
-        <f>LEFT(D7,FIND(".",D7,FIND(".",D7)+1)-1)&amp;".255.254"</f>
-        <v>10.33.255.254</v>
-      </c>
-      <c r="I7" s="14">
-        <v>40</v>
-      </c>
-      <c r="J7" s="14">
-        <v>42</v>
-      </c>
-      <c r="K7" s="14">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A8" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="B8" s="14">
-        <v>40</v>
-      </c>
-      <c r="C8" s="14">
-        <v>0</v>
-      </c>
-      <c r="D8" s="14" t="str">
-        <f>10&amp;"."&amp;(B8+A2)&amp;"."&amp;0&amp;"."&amp;0</f>
-        <v>10.43.0.0</v>
-      </c>
-      <c r="E8" s="14" t="str">
-        <f t="shared" si="0"/>
-        <v>10.43.0.1</v>
-      </c>
-      <c r="F8" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="G8" s="14" t="str">
-        <f t="shared" si="1"/>
-        <v>10.43.0.1</v>
-      </c>
-      <c r="H8" s="14" t="str">
-        <f>LEFT(D8,FIND(".",D8,FIND(".",D8)+1)-1)&amp;".255.254"</f>
-        <v>10.43.255.254</v>
-      </c>
-      <c r="I8" s="14">
-        <v>40</v>
-      </c>
-      <c r="J8" s="14">
-        <v>41</v>
-      </c>
-      <c r="K8" s="14">
+      <c r="B11" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="C11" s="13">
         <v>10</v>
       </c>
-    </row>
-    <row r="9" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A9" s="14"/>
-      <c r="B9" s="14"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
-      <c r="H9" s="14"/>
-      <c r="I9" s="14"/>
-      <c r="J9" s="14"/>
-      <c r="K9" s="14"/>
-    </row>
-    <row r="10" spans="1:12" ht="15" x14ac:dyDescent="0.2">
-      <c r="A10" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="D10" s="14" t="s">
-        <v>37</v>
-      </c>
-      <c r="E10" s="14"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="14"/>
-      <c r="H10" s="14"/>
-      <c r="I10" s="14"/>
-      <c r="J10" s="14"/>
-      <c r="K10" s="14"/>
-      <c r="L10" s="14"/>
-    </row>
-    <row r="11" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A11" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="B11" s="18" t="s">
-        <v>38</v>
-      </c>
-      <c r="C11" s="14">
-        <v>10</v>
-      </c>
-      <c r="D11" s="14" t="str">
+      <c r="D11" s="13" t="str">
         <f>A2&amp;"."&amp;A2&amp;"."&amp;A2&amp;"."&amp;(C11)</f>
         <v>3.3.3.10</v>
       </c>
-      <c r="E11" s="14"/>
-      <c r="F11" s="14"/>
-      <c r="G11" s="14"/>
-      <c r="H11" s="14"/>
-      <c r="I11" s="14"/>
-      <c r="J11" s="14"/>
-      <c r="K11" s="14"/>
-      <c r="L11" s="14"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="13"/>
+      <c r="G11" s="13"/>
+      <c r="H11" s="13"/>
+      <c r="I11" s="13"/>
+      <c r="J11" s="13"/>
+      <c r="K11" s="13"/>
+      <c r="L11" s="13"/>
     </row>
     <row r="12" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A12" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="B12" s="18" t="s">
-        <v>39</v>
-      </c>
-      <c r="C12" s="14">
+      <c r="A12" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="B12" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" s="13">
         <v>20</v>
       </c>
-      <c r="D12" s="14" t="str">
+      <c r="D12" s="13" t="str">
         <f>A2&amp;"."&amp;A2&amp;"."&amp;A2&amp;"."&amp;(C12)</f>
         <v>3.3.3.20</v>
       </c>
-      <c r="E12" s="14"/>
-      <c r="F12" s="14"/>
-      <c r="G12" s="14"/>
-      <c r="H12" s="14"/>
-      <c r="I12" s="14"/>
-      <c r="J12" s="14"/>
-      <c r="K12" s="14"/>
-      <c r="L12" s="14"/>
+      <c r="E12" s="13"/>
+      <c r="F12" s="13"/>
+      <c r="G12" s="13"/>
+      <c r="H12" s="13"/>
+      <c r="I12" s="13"/>
+      <c r="J12" s="13"/>
+      <c r="K12" s="13"/>
+      <c r="L12" s="13"/>
     </row>
     <row r="13" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A13" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="B13" s="18" t="s">
-        <v>40</v>
-      </c>
-      <c r="C13" s="14">
+      <c r="A13" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="B13" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="C13" s="13">
         <v>30</v>
       </c>
-      <c r="D13" s="14" t="str">
+      <c r="D13" s="13" t="str">
         <f>A2&amp;"."&amp;A2&amp;"."&amp;A2&amp;"."&amp;(C13)</f>
         <v>3.3.3.30</v>
       </c>
-      <c r="E13" s="14"/>
-      <c r="F13" s="14"/>
-      <c r="G13" s="14"/>
-      <c r="H13" s="14"/>
-      <c r="I13" s="14"/>
-      <c r="J13" s="14"/>
-      <c r="K13" s="14"/>
-      <c r="L13" s="14"/>
+      <c r="E13" s="13"/>
+      <c r="F13" s="13"/>
+      <c r="G13" s="13"/>
+      <c r="H13" s="13"/>
+      <c r="I13" s="13"/>
+      <c r="J13" s="13"/>
+      <c r="K13" s="13"/>
+      <c r="L13" s="13"/>
     </row>
     <row r="14" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A14" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="B14" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="C14" s="14">
+      <c r="A14" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="B14" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="D14" s="14" t="str">
+      <c r="C14" s="13">
+        <v>40</v>
+      </c>
+      <c r="D14" s="13" t="str">
         <f t="shared" ref="D14" si="2">$A$2&amp;"."&amp;$A$2&amp;"."&amp;$A$2&amp;"."&amp;(C14)</f>
         <v>3.3.3.40</v>
       </c>
-      <c r="E14" s="14"/>
-      <c r="F14" s="14"/>
-      <c r="G14" s="14"/>
-      <c r="H14" s="14"/>
-      <c r="I14" s="14"/>
-      <c r="J14" s="14"/>
-      <c r="K14" s="14"/>
-      <c r="L14" s="14"/>
+      <c r="E14" s="13"/>
+      <c r="F14" s="13"/>
+      <c r="G14" s="13"/>
+      <c r="H14" s="13"/>
+      <c r="I14" s="13"/>
+      <c r="J14" s="13"/>
+      <c r="K14" s="13"/>
+      <c r="L14" s="13"/>
     </row>
     <row r="15" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A15" s="14"/>
-      <c r="B15" s="14"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="14"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="14"/>
-      <c r="H15" s="14"/>
-      <c r="I15" s="14"/>
-      <c r="J15" s="14"/>
-      <c r="K15" s="14"/>
+      <c r="A15" s="13"/>
+      <c r="B15" s="13"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="13"/>
+      <c r="H15" s="13"/>
+      <c r="I15" s="13"/>
+      <c r="J15" s="13"/>
+      <c r="K15" s="13"/>
     </row>
     <row r="16" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A16" s="14" t="s">
+      <c r="A16" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="B16" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="C16" s="14" t="s">
+      <c r="D16" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="E16" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="D16" s="14" t="s">
-        <v>24</v>
-      </c>
-      <c r="E16" s="14" t="s">
+      <c r="F16" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="F16" s="14" t="s">
+      <c r="G16" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="G16" s="14" t="s">
+      <c r="H16" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="H16" s="14" t="s">
+      <c r="I16" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="I16" s="14" t="s">
+      <c r="J16" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="J16" s="14" t="s">
+      <c r="K16" s="13"/>
+    </row>
+    <row r="17" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A17" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="K16" s="14"/>
-    </row>
-    <row r="17" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A17" s="14" t="s">
-        <v>50</v>
-      </c>
-      <c r="B17" s="14" t="s">
+      <c r="B17" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="C17" s="14" t="str">
+      <c r="C17" s="13" t="str">
         <f>172&amp;"."&amp;16&amp;"."&amp;0&amp;"."&amp;(H17+$A$2)</f>
         <v>172.16.0.13</v>
       </c>
-      <c r="D17" s="14" t="s">
+      <c r="D17" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="E17" s="13"/>
+      <c r="F17" s="13"/>
+      <c r="G17" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="E17" s="14"/>
-      <c r="F17" s="14"/>
-      <c r="G17" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="H17" s="14">
+      <c r="H17" s="13">
         <v>10</v>
       </c>
-      <c r="I17" s="14">
+      <c r="I17" s="13">
         <f t="array" ref="I17">'Site 1 (HUB)'!I17</f>
         <v>0</v>
       </c>
-      <c r="J17" s="14"/>
-      <c r="K17" s="14"/>
+      <c r="J17" s="13"/>
+      <c r="K17" s="13"/>
     </row>
     <row r="18" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A18" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="B18" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="C18" s="14" t="str">
+      <c r="A18" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="C18" s="13" t="str">
         <f>172&amp;"."&amp;16&amp;"."&amp;0&amp;"."&amp;(H18+$A$2)</f>
         <v>172.16.0.33</v>
       </c>
-      <c r="D18" s="14" t="s">
+      <c r="D18" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="E18" s="13"/>
+      <c r="F18" s="13"/>
+      <c r="G18" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="E18" s="14"/>
-      <c r="F18" s="14"/>
-      <c r="G18" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="H18" s="14">
+      <c r="H18" s="13">
         <v>30</v>
       </c>
-      <c r="I18" s="14" t="b">
+      <c r="I18" s="13" t="b">
         <f t="array" ref="I18">'Site 1 (HUB)'!I18</f>
         <v>1</v>
       </c>
-      <c r="J18" s="14"/>
-      <c r="K18" s="14"/>
+      <c r="J18" s="13"/>
+      <c r="K18" s="13"/>
     </row>
     <row r="19" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A19" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="B19" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="C19" s="14" t="str">
+      <c r="A19" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="C19" s="13" t="str">
         <f t="shared" ref="C19" si="3">172&amp;"."&amp;16&amp;"."&amp;0&amp;"."&amp;(H19+$A$2)</f>
         <v>172.16.0.43</v>
       </c>
-      <c r="D19" s="14" t="s">
+      <c r="D19" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="E19" s="13"/>
+      <c r="F19" s="13"/>
+      <c r="G19" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="E19" s="14"/>
-      <c r="F19" s="14"/>
-      <c r="G19" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="H19" s="14">
+      <c r="H19" s="13">
         <v>40</v>
       </c>
-      <c r="I19" s="14" t="b">
+      <c r="I19" s="13" t="b">
         <f>'Site 1 (HUB)'!I19</f>
         <v>1</v>
       </c>
-      <c r="J19" s="14"/>
-      <c r="K19" s="14"/>
+      <c r="J19" s="13"/>
+      <c r="K19" s="13"/>
     </row>
     <row r="20" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A20" s="14"/>
-      <c r="B20" s="14"/>
-      <c r="C20" s="14"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14"/>
-      <c r="F20" s="14"/>
-      <c r="G20" s="14"/>
-      <c r="H20" s="14"/>
-      <c r="I20" s="14"/>
-      <c r="J20" s="14"/>
-      <c r="K20" s="14"/>
+      <c r="A20" s="13"/>
+      <c r="B20" s="13"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="13"/>
+      <c r="F20" s="13"/>
+      <c r="G20" s="13"/>
+      <c r="H20" s="13"/>
+      <c r="I20" s="13"/>
+      <c r="J20" s="13"/>
+      <c r="K20" s="13"/>
     </row>
     <row r="21" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A21" s="14" t="s">
+      <c r="A21" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B21" s="14" t="s">
+      <c r="B21" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="C21" s="14" t="s">
+      <c r="C21" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="D21" s="14" t="s">
+      <c r="D21" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="E21" s="14" t="s">
+      <c r="E21" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="F21" s="14" t="s">
+      <c r="F21" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="G21" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="G21" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="H21" s="14"/>
-      <c r="I21" s="14"/>
-      <c r="J21" s="14"/>
-      <c r="K21" s="14"/>
+      <c r="H21" s="13"/>
+      <c r="I21" s="13"/>
+      <c r="J21" s="13"/>
+      <c r="K21" s="13"/>
     </row>
     <row r="22" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A22" s="14">
+      <c r="A22" s="13">
         <f>A2</f>
         <v>3</v>
       </c>
-      <c r="B22" s="14" t="s">
+      <c r="B22" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="C22" s="14" t="s">
+      <c r="C22" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="D22" s="14" t="s">
+      <c r="D22" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="E22" s="14" t="s">
+      <c r="E22" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="F22" s="14">
+      <c r="F22" s="13">
         <v>2</v>
       </c>
       <c r="G22" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="H22" s="20"/>
+      <c r="I22" s="13"/>
+      <c r="J22" s="13"/>
+      <c r="K22" s="13"/>
+    </row>
+    <row r="23" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A23" s="13"/>
+      <c r="B23" s="13"/>
+      <c r="C23" s="13"/>
+      <c r="D23" s="13"/>
+      <c r="E23" s="13"/>
+      <c r="F23" s="13"/>
+      <c r="G23" s="13"/>
+      <c r="H23" s="13"/>
+      <c r="I23" s="13"/>
+      <c r="J23" s="13"/>
+      <c r="K23" s="13"/>
+    </row>
+    <row r="24" spans="1:12" ht="15" x14ac:dyDescent="0.2">
+      <c r="A24" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="H22" s="21"/>
-      <c r="I22" s="14"/>
-      <c r="J22" s="14"/>
-      <c r="K22" s="14"/>
-    </row>
-    <row r="23" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A23" s="14"/>
-      <c r="B23" s="14"/>
-      <c r="C23" s="14"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="14"/>
-      <c r="F23" s="14"/>
-      <c r="G23" s="14"/>
-      <c r="H23" s="14"/>
-      <c r="I23" s="14"/>
-      <c r="J23" s="14"/>
-      <c r="K23" s="14"/>
-    </row>
-    <row r="24" spans="1:12" ht="15" x14ac:dyDescent="0.2">
-      <c r="A24" s="15" t="s">
+      <c r="B24" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="B24" s="15" t="s">
+      <c r="C24" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="C24" s="15" t="s">
+      <c r="D24" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="E24" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="F24" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="D24" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="E24" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="F24" s="15" t="s">
+      <c r="G24" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="G24" s="15" t="s">
+      <c r="H24" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="H24" s="15" t="s">
+      <c r="I24" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="I24" s="15" t="s">
+      <c r="J24" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="K24" s="14" t="s">
         <v>64</v>
       </c>
-      <c r="J24" s="15" t="s">
-        <v>1</v>
-      </c>
-      <c r="K24" s="15" t="s">
+      <c r="L24" t="s">
         <v>65</v>
       </c>
-      <c r="L24" t="s">
-        <v>66</v>
-      </c>
     </row>
     <row r="25" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A25" s="8">
+      <c r="A25" s="7">
         <f>(ROW())-(ROW()-1)</f>
         <v>1</v>
       </c>
-      <c r="B25" s="8">
+      <c r="B25" s="7">
         <v>10</v>
       </c>
-      <c r="C25" s="8" t="str">
+      <c r="C25" s="7" t="str">
         <f>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A25)</f>
-        <v>10.13.0.2</v>
-      </c>
-      <c r="D25" s="8" t="str">
+        <v>10.3.10.2</v>
+      </c>
+      <c r="D25" s="7" t="str">
         <f>$E$5</f>
-        <v>10.13.0.1</v>
-      </c>
-      <c r="E25" s="8" t="str">
+        <v>10.3.10.1</v>
+      </c>
+      <c r="E25" s="7" t="str">
         <f>$F$5</f>
-        <v>255.255.0.0</v>
-      </c>
-      <c r="F25" s="8">
+        <v>255.255.255.0</v>
+      </c>
+      <c r="F25" s="7">
         <v>24</v>
       </c>
-      <c r="G25" s="8">
+      <c r="G25" s="7">
         <v>1</v>
       </c>
-      <c r="H25" s="11">
+      <c r="H25" s="10">
         <v>0</v>
       </c>
-      <c r="I25" s="8" t="s">
-        <v>67</v>
+      <c r="I25" s="7" t="s">
+        <v>66</v>
       </c>
       <c r="J25" s="2" t="s">
         <v>12</v>
@@ -6493,23 +6448,19 @@
         <f>IF($A25=1,F25-G25-H25*$F$22-2-IF(OR(UPPER($G$22)="SPAN",UPPER($G$22)="RSPAN"),1,0),F25-G25-(1+H25)*$F$22-1)</f>
         <v>20</v>
       </c>
-      <c r="L25" t="str">
-        <f>10&amp;"."&amp;(50+$A$2)&amp;"."&amp;0&amp;"."&amp;(A25+1)</f>
-        <v>10.53.0.2</v>
-      </c>
     </row>
     <row r="26" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A26" s="14"/>
-      <c r="B26" s="14"/>
-      <c r="C26" s="14"/>
-      <c r="D26" s="14"/>
-      <c r="E26" s="14"/>
-      <c r="F26" s="14"/>
-      <c r="G26" s="14"/>
-      <c r="H26" s="14"/>
-      <c r="I26" s="14"/>
-      <c r="J26" s="14"/>
-      <c r="K26" s="14"/>
+      <c r="A26" s="13"/>
+      <c r="B26" s="13"/>
+      <c r="C26" s="13"/>
+      <c r="D26" s="13"/>
+      <c r="E26" s="13"/>
+      <c r="F26" s="13"/>
+      <c r="G26" s="13"/>
+      <c r="H26" s="13"/>
+      <c r="I26" s="13"/>
+      <c r="J26" s="13"/>
+      <c r="K26" s="13"/>
     </row>
   </sheetData>
   <dataValidations count="3">
@@ -6550,278 +6501,278 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="25" t="s">
-        <v>45</v>
-      </c>
-      <c r="C1" s="25" t="s">
+      <c r="C1" s="24" t="s">
+        <v>69</v>
+      </c>
+      <c r="D1" s="24" t="s">
         <v>70</v>
       </c>
-      <c r="D1" s="25" t="s">
+      <c r="E1" s="24" t="s">
         <v>71</v>
       </c>
-      <c r="E1" s="25" t="s">
+      <c r="G1" s="26" t="s">
         <v>72</v>
       </c>
-      <c r="G1" s="27" t="s">
+      <c r="H1" s="26" t="s">
         <v>73</v>
       </c>
-      <c r="H1" s="27" t="s">
+    </row>
+    <row r="2" spans="1:8" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A2" s="25" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2" s="25" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="25" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A2" s="26" t="s">
+      <c r="D2" s="25">
+        <v>67</v>
+      </c>
+      <c r="E2" s="25" t="s">
+        <v>75</v>
+      </c>
+      <c r="G2" s="27" t="s">
+        <v>76</v>
+      </c>
+      <c r="H2" s="27" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A3" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="B2" s="26" t="s">
+      <c r="B3" s="25" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" s="25" t="s">
+        <v>78</v>
+      </c>
+      <c r="D3" s="25" t="s">
+        <v>79</v>
+      </c>
+      <c r="E3" s="25" t="s">
+        <v>75</v>
+      </c>
+      <c r="G3" s="27" t="s">
+        <v>80</v>
+      </c>
+      <c r="H3" s="27" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A4" s="25" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="26" t="s">
+      <c r="C4" s="25" t="s">
+        <v>74</v>
+      </c>
+      <c r="D4" s="25">
+        <v>67</v>
+      </c>
+      <c r="E4" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="D2" s="26">
+      <c r="G4" s="27" t="s">
+        <v>82</v>
+      </c>
+      <c r="H4" s="27" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A5" s="25" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" s="25" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" s="25" t="s">
+        <v>78</v>
+      </c>
+      <c r="D5" s="25" t="s">
+        <v>79</v>
+      </c>
+      <c r="E5" s="25" t="s">
+        <v>84</v>
+      </c>
+      <c r="G5" s="27" t="s">
+        <v>8</v>
+      </c>
+      <c r="H5" s="27" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A6" s="25" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="25" t="s">
+        <v>86</v>
+      </c>
+      <c r="C6" s="25" t="s">
+        <v>74</v>
+      </c>
+      <c r="D6" s="25">
+        <v>53</v>
+      </c>
+      <c r="E6" s="25" t="s">
+        <v>75</v>
+      </c>
+      <c r="G6" s="27" t="s">
+        <v>87</v>
+      </c>
+      <c r="H6" s="27" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A7" s="25" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" s="25" t="s">
+        <v>86</v>
+      </c>
+      <c r="C7" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="D7" s="25">
+        <v>53</v>
+      </c>
+      <c r="E7" s="25" t="s">
+        <v>75</v>
+      </c>
+      <c r="G7" s="27" t="s">
+        <v>90</v>
+      </c>
+      <c r="H7" s="27" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A8" s="25" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" s="25" t="s">
+        <v>92</v>
+      </c>
+      <c r="C8" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="D8" s="25">
+        <v>80</v>
+      </c>
+      <c r="E8" s="25" t="s">
+        <v>75</v>
+      </c>
+      <c r="G8" s="27" t="s">
+        <v>93</v>
+      </c>
+      <c r="H8" s="27" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A9" s="25" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" s="25" t="s">
+        <v>92</v>
+      </c>
+      <c r="C9" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="D9" s="25">
+        <v>443</v>
+      </c>
+      <c r="E9" s="25" t="s">
+        <v>75</v>
+      </c>
+      <c r="G9" s="27" t="s">
+        <v>95</v>
+      </c>
+      <c r="H9" s="27" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A10" s="25" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" s="25" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="25" t="s">
+        <v>74</v>
+      </c>
+      <c r="D10" s="25">
         <v>67</v>
       </c>
-      <c r="E2" s="26" t="s">
-        <v>76</v>
-      </c>
-      <c r="G2" s="28" t="s">
-        <v>77</v>
-      </c>
-      <c r="H2" s="28" t="s">
+      <c r="E10" s="25" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A11" s="25" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" s="25" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11" s="25" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A3" s="26" t="s">
-        <v>30</v>
-      </c>
-      <c r="B3" s="26" t="s">
-        <v>30</v>
-      </c>
-      <c r="C3" s="26" t="s">
+      <c r="D11" s="25" t="s">
         <v>79</v>
       </c>
-      <c r="D3" s="26" t="s">
-        <v>80</v>
-      </c>
-      <c r="E3" s="26" t="s">
-        <v>76</v>
-      </c>
-      <c r="G3" s="28" t="s">
-        <v>81</v>
-      </c>
-      <c r="H3" s="28" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A4" s="26" t="s">
-        <v>32</v>
-      </c>
-      <c r="B4" s="26" t="s">
+      <c r="E11" s="25" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A12" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="B12" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="26" t="s">
+      <c r="C12" s="25" t="s">
+        <v>74</v>
+      </c>
+      <c r="D12" s="25">
+        <v>67</v>
+      </c>
+      <c r="E12" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="D4" s="26">
-        <v>67</v>
-      </c>
-      <c r="E4" s="26" t="s">
-        <v>76</v>
-      </c>
-      <c r="G4" s="28" t="s">
-        <v>83</v>
-      </c>
-      <c r="H4" s="28" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A5" s="26" t="s">
-        <v>32</v>
-      </c>
-      <c r="B5" s="26" t="s">
-        <v>32</v>
-      </c>
-      <c r="C5" s="26" t="s">
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A13" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="B13" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="C13" s="25" t="s">
+        <v>78</v>
+      </c>
+      <c r="D13" s="25" t="s">
         <v>79</v>
       </c>
-      <c r="D5" s="26" t="s">
-        <v>80</v>
-      </c>
-      <c r="E5" s="26" t="s">
-        <v>85</v>
-      </c>
-      <c r="G5" s="28" t="s">
-        <v>8</v>
-      </c>
-      <c r="H5" s="28" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A6" s="26" t="s">
-        <v>32</v>
-      </c>
-      <c r="B6" s="26" t="s">
-        <v>87</v>
-      </c>
-      <c r="C6" s="26" t="s">
+      <c r="E13" s="25" t="s">
         <v>75</v>
-      </c>
-      <c r="D6" s="26">
-        <v>53</v>
-      </c>
-      <c r="E6" s="26" t="s">
-        <v>76</v>
-      </c>
-      <c r="G6" s="28" t="s">
-        <v>88</v>
-      </c>
-      <c r="H6" s="28" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A7" s="26" t="s">
-        <v>32</v>
-      </c>
-      <c r="B7" s="26" t="s">
-        <v>87</v>
-      </c>
-      <c r="C7" s="26" t="s">
-        <v>90</v>
-      </c>
-      <c r="D7" s="26">
-        <v>53</v>
-      </c>
-      <c r="E7" s="26" t="s">
-        <v>76</v>
-      </c>
-      <c r="G7" s="28" t="s">
-        <v>91</v>
-      </c>
-      <c r="H7" s="28" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A8" s="26" t="s">
-        <v>32</v>
-      </c>
-      <c r="B8" s="26" t="s">
-        <v>93</v>
-      </c>
-      <c r="C8" s="26" t="s">
-        <v>90</v>
-      </c>
-      <c r="D8" s="26">
-        <v>80</v>
-      </c>
-      <c r="E8" s="26" t="s">
-        <v>76</v>
-      </c>
-      <c r="G8" s="28" t="s">
-        <v>94</v>
-      </c>
-      <c r="H8" s="28" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A9" s="26" t="s">
-        <v>32</v>
-      </c>
-      <c r="B9" s="26" t="s">
-        <v>93</v>
-      </c>
-      <c r="C9" s="26" t="s">
-        <v>90</v>
-      </c>
-      <c r="D9" s="26">
-        <v>443</v>
-      </c>
-      <c r="E9" s="26" t="s">
-        <v>76</v>
-      </c>
-      <c r="G9" s="28" t="s">
-        <v>96</v>
-      </c>
-      <c r="H9" s="28" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A10" s="26" t="s">
-        <v>33</v>
-      </c>
-      <c r="B10" s="26" t="s">
-        <v>8</v>
-      </c>
-      <c r="C10" s="26" t="s">
-        <v>75</v>
-      </c>
-      <c r="D10" s="26">
-        <v>67</v>
-      </c>
-      <c r="E10" s="26" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A11" s="26" t="s">
-        <v>33</v>
-      </c>
-      <c r="B11" s="26" t="s">
-        <v>33</v>
-      </c>
-      <c r="C11" s="26" t="s">
-        <v>79</v>
-      </c>
-      <c r="D11" s="26" t="s">
-        <v>80</v>
-      </c>
-      <c r="E11" s="26" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A12" s="26" t="s">
-        <v>34</v>
-      </c>
-      <c r="B12" s="26" t="s">
-        <v>8</v>
-      </c>
-      <c r="C12" s="26" t="s">
-        <v>75</v>
-      </c>
-      <c r="D12" s="26">
-        <v>67</v>
-      </c>
-      <c r="E12" s="26" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A13" s="26" t="s">
-        <v>34</v>
-      </c>
-      <c r="B13" s="26" t="s">
-        <v>34</v>
-      </c>
-      <c r="C13" s="26" t="s">
-        <v>79</v>
-      </c>
-      <c r="D13" s="26" t="s">
-        <v>80</v>
-      </c>
-      <c r="E13" s="26" t="s">
-        <v>76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>